<commit_message>
Refresh deck and workbook for operational audiences
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rae47614331d24053"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="Rfafa0be55547472f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4bbf4d136fcd4b9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R36267d3954da4346"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rc3da8799cb924929"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -17,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="21">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -108,8 +109,36 @@
       <x:color rgb="FF155E4A"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFD52B1E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFD52B1E"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -144,6 +173,46 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFFF1D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -203,7 +272,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="74">
+  <x:cellXfs count="116">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -374,6 +443,112 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="200" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -387,7 +562,7 @@
         <x:color rgb="FF155E4A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF4E7"/>
         </x:patternFill>
       </x:fill>
@@ -602,37 +777,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="100" t="str">
         <x:v>Synthetic Reliability Report</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
+      <x:c r="B1" s="100"/>
+      <x:c r="C1" s="100"/>
+      <x:c r="D1" s="100"/>
+      <x:c r="E1" s="100"/>
+      <x:c r="F1" s="100"/>
+      <x:c r="G1" s="100"/>
       <x:c r="H1" s="43"/>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="43"/>
-      <x:c r="B2" s="43"/>
-      <x:c r="C2" s="43"/>
-      <x:c r="D2" s="43"/>
-      <x:c r="E2" s="43"/>
-      <x:c r="F2" s="43"/>
-      <x:c r="G2" s="43"/>
+      <x:c r="A2" s="100"/>
+      <x:c r="B2" s="100"/>
+      <x:c r="C2" s="100"/>
+      <x:c r="D2" s="100"/>
+      <x:c r="E2" s="100"/>
+      <x:c r="F2" s="100"/>
+      <x:c r="G2" s="100"/>
       <x:c r="H2" s="43"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="44" t="str">
+      <x:c r="A3" s="101" t="str">
         <x:v>Portfolio demonstration only - generalized architecture, synthetic values, no production connection</x:v>
       </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
+      <x:c r="B3" s="101"/>
+      <x:c r="C3" s="101"/>
+      <x:c r="D3" s="101"/>
+      <x:c r="E3" s="101"/>
+      <x:c r="F3" s="101"/>
+      <x:c r="G3" s="101"/>
       <x:c r="H3" s="44"/>
     </x:row>
     <x:row r="4">
@@ -646,19 +821,19 @@
       <x:c r="H4" s="45"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="46" t="str">
+      <x:c r="A5" s="102" t="str">
         <x:v>Total governed writes</x:v>
       </x:c>
-      <x:c r="B5" s="46" t="str"/>
-      <x:c r="C5" s="46" t="str">
+      <x:c r="B5" s="102" t="str"/>
+      <x:c r="C5" s="102" t="str">
         <x:v>Equivalent replay writes</x:v>
       </x:c>
-      <x:c r="D5" s="46" t="str"/>
-      <x:c r="E5" s="46" t="str">
+      <x:c r="D5" s="102" t="str"/>
+      <x:c r="E5" s="102" t="str">
         <x:v>Final remote version</x:v>
       </x:c>
-      <x:c r="F5" s="46" t="str"/>
-      <x:c r="G5" s="46" t="str">
+      <x:c r="F5" s="102" t="str"/>
+      <x:c r="G5" s="102" t="str">
         <x:v>Overlapping writers</x:v>
       </x:c>
       <x:c r="H5" s="46" t="str"/>
@@ -706,33 +881,33 @@
       <x:c r="H8" s="45"/>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="51" t="str">
+      <x:c r="A9" s="103" t="str">
         <x:v>Reliability controls demonstrated</x:v>
       </x:c>
-      <x:c r="B9" s="51"/>
-      <x:c r="C9" s="51"/>
-      <x:c r="D9" s="51"/>
-      <x:c r="E9" s="51"/>
-      <x:c r="F9" s="51"/>
-      <x:c r="G9" s="51"/>
+      <x:c r="B9" s="103"/>
+      <x:c r="C9" s="103"/>
+      <x:c r="D9" s="103"/>
+      <x:c r="E9" s="103"/>
+      <x:c r="F9" s="103"/>
+      <x:c r="G9" s="103"/>
       <x:c r="H9" s="51"/>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="46" t="str">
+      <x:c r="A10" s="102" t="str">
         <x:v>Invariant</x:v>
       </x:c>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="B10" s="102" t="str">
         <x:v>Mechanism</x:v>
       </x:c>
-      <x:c r="C10" s="46" t="str">
+      <x:c r="C10" s="102" t="str">
         <x:v>Synthetic result</x:v>
       </x:c>
-      <x:c r="D10" s="46" t="str">
+      <x:c r="D10" s="102" t="str">
         <x:v>Boundary</x:v>
       </x:c>
-      <x:c r="E10" s="46" t="str"/>
-      <x:c r="F10" s="46" t="str"/>
-      <x:c r="G10" s="46" t="str"/>
+      <x:c r="E10" s="102" t="str"/>
+      <x:c r="F10" s="102" t="str"/>
+      <x:c r="G10" s="102" t="str"/>
       <x:c r="H10" s="46" t="str"/>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
@@ -742,7 +917,7 @@
       <x:c r="B11" s="52" t="str">
         <x:v>Governed material identity</x:v>
       </x:c>
-      <x:c r="C11" s="53" t="str">
+      <x:c r="C11" s="78" t="str">
         <x:v>Exact no-op / zero writes</x:v>
       </x:c>
       <x:c r="D11" s="52" t="str">
@@ -760,7 +935,7 @@
       <x:c r="B12" s="54" t="str">
         <x:v>Retained candidate plus GET</x:v>
       </x:c>
-      <x:c r="C12" s="55" t="str">
+      <x:c r="C12" s="79" t="str">
         <x:v>Settled / zero retry writes</x:v>
       </x:c>
       <x:c r="D12" s="54" t="str">
@@ -778,7 +953,7 @@
       <x:c r="B13" s="52" t="str">
         <x:v>Durable expected output</x:v>
       </x:c>
-      <x:c r="C13" s="53" t="str">
+      <x:c r="C13" s="78" t="str">
         <x:v>Same item advanced once</x:v>
       </x:c>
       <x:c r="D13" s="52" t="str">
@@ -796,7 +971,7 @@
       <x:c r="B14" s="54" t="str">
         <x:v>Exclusive writer lease</x:v>
       </x:c>
-      <x:c r="C14" s="55" t="str">
+      <x:c r="C14" s="79" t="str">
         <x:v>Second writer refused</x:v>
       </x:c>
       <x:c r="D14" s="54" t="str">
@@ -814,7 +989,7 @@
       <x:c r="B15" s="52" t="str">
         <x:v>Immutable prior release</x:v>
       </x:c>
-      <x:c r="C15" s="53" t="str">
+      <x:c r="C15" s="78" t="str">
         <x:v>Exact rollback restored</x:v>
       </x:c>
       <x:c r="D15" s="52" t="str">
@@ -836,15 +1011,15 @@
       <x:c r="H16" s="45"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
-      <x:c r="A17" s="56" t="str">
+      <x:c r="A17" s="104" t="str">
         <x:v>Claim boundary: this workbook demonstrates reliability behavior only; it does not represent production data, financial impact, or blanket accuracy.</x:v>
       </x:c>
-      <x:c r="B17" s="56"/>
-      <x:c r="C17" s="56"/>
-      <x:c r="D17" s="56"/>
-      <x:c r="E17" s="56"/>
-      <x:c r="F17" s="56"/>
-      <x:c r="G17" s="56"/>
+      <x:c r="B17" s="104"/>
+      <x:c r="C17" s="104"/>
+      <x:c r="D17" s="104"/>
+      <x:c r="E17" s="104"/>
+      <x:c r="F17" s="104"/>
+      <x:c r="G17" s="104"/>
       <x:c r="H17" s="56"/>
     </x:row>
   </x:sheetData>
@@ -888,31 +1063,31 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="59" t="str">
+      <x:c r="A1" s="105" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="B1" s="59" t="str">
+      <x:c r="B1" s="105" t="str">
         <x:v>Event</x:v>
       </x:c>
-      <x:c r="C1" s="59" t="str">
+      <x:c r="C1" s="105" t="str">
         <x:v>State</x:v>
       </x:c>
-      <x:c r="D1" s="59" t="str">
+      <x:c r="D1" s="105" t="str">
         <x:v>Material</x:v>
       </x:c>
-      <x:c r="E1" s="59" t="str">
+      <x:c r="E1" s="105" t="str">
         <x:v>Remote version</x:v>
       </x:c>
-      <x:c r="F1" s="59" t="str">
+      <x:c r="F1" s="105" t="str">
         <x:v>Writes</x:v>
       </x:c>
-      <x:c r="G1" s="59" t="str">
+      <x:c r="G1" s="105" t="str">
         <x:v>Settlement</x:v>
       </x:c>
-      <x:c r="H1" s="59" t="str">
+      <x:c r="H1" s="105" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="I1" s="59" t="str">
+      <x:c r="I1" s="105" t="str">
         <x:v>Writer overlap</x:v>
       </x:c>
     </x:row>
@@ -975,31 +1150,31 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="72" t="n">
+      <x:c r="A4" s="108" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="68" t="str">
+      <x:c r="B4" s="109" t="str">
         <x:v>Equivalent capture marker changes</x:v>
       </x:c>
-      <x:c r="C4" s="68" t="str">
+      <x:c r="C4" s="109" t="str">
         <x:v>certified</x:v>
       </x:c>
-      <x:c r="D4" s="68" t="str">
+      <x:c r="D4" s="109" t="str">
         <x:v>material-a</x:v>
       </x:c>
-      <x:c r="E4" s="72" t="n">
+      <x:c r="E4" s="108" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" s="72" t="n">
+      <x:c r="F4" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G4" s="68" t="str">
+      <x:c r="G4" s="109" t="str">
         <x:v>exact GET</x:v>
       </x:c>
-      <x:c r="H4" s="68" t="str">
+      <x:c r="H4" s="109" t="str">
         <x:v>exact no-op</x:v>
       </x:c>
-      <x:c r="I4" s="72" t="n">
+      <x:c r="I4" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1033,31 +1208,31 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="72" t="n">
+      <x:c r="A6" s="108" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="68" t="str">
+      <x:c r="B6" s="109" t="str">
         <x:v>Equivalent replay after settlement</x:v>
       </x:c>
-      <x:c r="C6" s="68" t="str">
+      <x:c r="C6" s="109" t="str">
         <x:v>certified</x:v>
       </x:c>
-      <x:c r="D6" s="68" t="str">
+      <x:c r="D6" s="109" t="str">
         <x:v>material-b</x:v>
       </x:c>
-      <x:c r="E6" s="72" t="n">
+      <x:c r="E6" s="108" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F6" s="72" t="n">
+      <x:c r="F6" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G6" s="68" t="str">
+      <x:c r="G6" s="109" t="str">
         <x:v>exact GET</x:v>
       </x:c>
-      <x:c r="H6" s="68" t="str">
+      <x:c r="H6" s="109" t="str">
         <x:v>exact no-op</x:v>
       </x:c>
-      <x:c r="I6" s="72" t="n">
+      <x:c r="I6" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1098,4 +1273,246 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="110" t="str">
+        <x:v>Prepared outputs for human review and action</x:v>
+      </x:c>
+      <x:c r="B1" s="110"/>
+      <x:c r="C1" s="110"/>
+      <x:c r="D1" s="110"/>
+      <x:c r="E1" s="110"/>
+      <x:c r="F1" s="110"/>
+      <x:c r="G1" s="110"/>
+      <x:c r="H1" s="110"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="110"/>
+      <x:c r="B2" s="110"/>
+      <x:c r="C2" s="110"/>
+      <x:c r="D2" s="110"/>
+      <x:c r="E2" s="110"/>
+      <x:c r="F2" s="110"/>
+      <x:c r="G2" s="110"/>
+      <x:c r="H2" s="110"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="111" t="str">
+        <x:v>Synthetic portfolio guide — no production connection; the platform supports decisions and does not make them.</x:v>
+      </x:c>
+      <x:c r="B3" s="111"/>
+      <x:c r="C3" s="111"/>
+      <x:c r="D3" s="111"/>
+      <x:c r="E3" s="111"/>
+      <x:c r="F3" s="111"/>
+      <x:c r="G3" s="111"/>
+      <x:c r="H3" s="111"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="112" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="B5" s="112" t="str"/>
+      <x:c r="C5" s="112" t="str">
+        <x:v>PRIMARY USER</x:v>
+      </x:c>
+      <x:c r="D5" s="112" t="str"/>
+      <x:c r="E5" s="112" t="str">
+        <x:v>WHAT AUTOMATION PREPARES</x:v>
+      </x:c>
+      <x:c r="F5" s="112" t="str"/>
+      <x:c r="G5" s="112" t="str">
+        <x:v>HUMAN USE</x:v>
+      </x:c>
+      <x:c r="H5" s="112" t="str"/>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="113" t="str">
+        <x:v>Shift Drafts</x:v>
+      </x:c>
+      <x:c r="B6" s="113" t="str"/>
+      <x:c r="C6" s="113" t="str">
+        <x:v>Supervisors</x:v>
+      </x:c>
+      <x:c r="D6" s="113" t="str"/>
+      <x:c r="E6" s="113" t="str">
+        <x:v>Collection, reconciliation, organization, spreadsheet preparation</x:v>
+      </x:c>
+      <x:c r="F6" s="113" t="str"/>
+      <x:c r="G6" s="113" t="str">
+        <x:v>Review exceptions, add context, finalize</x:v>
+      </x:c>
+      <x:c r="H6" s="113" t="str"/>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="113" t="str">
+        <x:v>Daily Production Reports</x:v>
+      </x:c>
+      <x:c r="B7" s="113" t="str"/>
+      <x:c r="C7" s="113" t="str">
+        <x:v>Managers</x:v>
+      </x:c>
+      <x:c r="D7" s="113" t="str"/>
+      <x:c r="E7" s="113" t="str">
+        <x:v>Production, molding, labor, quality, plan attainment, downtime</x:v>
+      </x:c>
+      <x:c r="F7" s="113" t="str"/>
+      <x:c r="G7" s="113" t="str">
+        <x:v>Investigate constraints; prioritize staffing, plan, maintenance, or coordination follow-up</x:v>
+      </x:c>
+      <x:c r="H7" s="113" t="str"/>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="113" t="str">
+        <x:v>Weekly Production Reports</x:v>
+      </x:c>
+      <x:c r="B8" s="113" t="str"/>
+      <x:c r="C8" s="113" t="str">
+        <x:v>Managers / teams</x:v>
+      </x:c>
+      <x:c r="D8" s="113" t="str"/>
+      <x:c r="E8" s="113" t="str">
+        <x:v>Comparable period views and source-linked trends</x:v>
+      </x:c>
+      <x:c r="F8" s="113" t="str"/>
+      <x:c r="G8" s="113" t="str">
+        <x:v>Capacity and labor planning; process improvement; weekly reviews</x:v>
+      </x:c>
+      <x:c r="H8" s="113" t="str"/>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="113" t="str">
+        <x:v>Weekly Downtime Reports</x:v>
+      </x:c>
+      <x:c r="B9" s="113" t="str"/>
+      <x:c r="C9" s="113" t="str">
+        <x:v>Managers / maintenance</x:v>
+      </x:c>
+      <x:c r="D9" s="113" t="str"/>
+      <x:c r="E9" s="113" t="str">
+        <x:v>Recurring-versus-isolated event patterns and downtime evidence</x:v>
+      </x:c>
+      <x:c r="F9" s="113" t="str"/>
+      <x:c r="G9" s="113" t="str">
+        <x:v>Maintenance prioritization; meetings; shift handoffs</x:v>
+      </x:c>
+      <x:c r="H9" s="113" t="str"/>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="105" t="str">
+        <x:v>Operational input → ingestion → reconciliation and source linkage → validation → prepared output → human review → operational action</x:v>
+      </x:c>
+      <x:c r="B11" s="105"/>
+      <x:c r="C11" s="105"/>
+      <x:c r="D11" s="105"/>
+      <x:c r="E11" s="105"/>
+      <x:c r="F11" s="105"/>
+      <x:c r="G11" s="105"/>
+      <x:c r="H11" s="105"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="114" t="str">
+        <x:v>MEASURED ENGINEERING RESULTS</x:v>
+      </x:c>
+      <x:c r="B13" s="114"/>
+      <x:c r="C13" s="114"/>
+      <x:c r="D13" s="114"/>
+      <x:c r="E13" s="114" t="str">
+        <x:v>ESTIMATED / MODELED OPPORTUNITIES</x:v>
+      </x:c>
+      <x:c r="F13" s="114"/>
+      <x:c r="G13" s="114"/>
+      <x:c r="H13" s="114"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="115" t="str">
+        <x:v>94.6% fewer replay-processing rows
+86.6% smaller local PostgreSQL fixture footprint</x:v>
+      </x:c>
+      <x:c r="B14" s="115"/>
+      <x:c r="C14" s="115"/>
+      <x:c r="D14" s="115"/>
+      <x:c r="E14" s="115" t="str">
+        <x:v>~90% retrieval-time reduction; ~87% storage-cost reduction; 30 hours/week and ~$52K annual labor value; up to 227.5K widgets/~$205K contribution-margin opportunity — all under documented assumptions</x:v>
+      </x:c>
+      <x:c r="F14" s="115"/>
+      <x:c r="G14" s="115"/>
+      <x:c r="H14" s="115"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="115"/>
+      <x:c r="B15" s="115"/>
+      <x:c r="C15" s="115"/>
+      <x:c r="D15" s="115"/>
+      <x:c r="E15" s="115"/>
+      <x:c r="F15" s="115"/>
+      <x:c r="G15" s="115"/>
+      <x:c r="H15" s="115"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="115"/>
+      <x:c r="B16" s="115"/>
+      <x:c r="C16" s="115"/>
+      <x:c r="D16" s="115"/>
+      <x:c r="E16" s="115"/>
+      <x:c r="F16" s="115"/>
+      <x:c r="G16" s="115"/>
+      <x:c r="H16" s="115"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="111" t="str">
+        <x:v>Modeled figures are planning opportunities—not booked savings, realized margin, guaranteed outcomes, or blanket accuracy.</x:v>
+      </x:c>
+      <x:c r="B18" s="111"/>
+      <x:c r="C18" s="111"/>
+      <x:c r="D18" s="111"/>
+      <x:c r="E18" s="111"/>
+      <x:c r="F18" s="111"/>
+      <x:c r="G18" s="111"/>
+      <x:c r="H18" s="111"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="G7:H7"/>
+    <x:mergeCell ref="A8:B8"/>
+    <x:mergeCell ref="C8:D8"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="G8:H8"/>
+    <x:mergeCell ref="A9:B9"/>
+    <x:mergeCell ref="C9:D9"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="G9:H9"/>
+    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A13:D13"/>
+    <x:mergeCell ref="E13:H13"/>
+    <x:mergeCell ref="A14:D16"/>
+    <x:mergeCell ref="E14:H16"/>
+    <x:mergeCell ref="A18:H18"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Condense case study and clarify artifact roles
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4bbf4d136fcd4b9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R36267d3954da4346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rc3da8799cb924929"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Re1ba9bdb2f5842d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R55af15bb67c84264"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R92d81601b3df43d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +18,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="21">
+  <x:fonts count="22">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -137,8 +137,13 @@
       <x:color rgb="FFD52B1E"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="14"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="16">
+  <x:fills count="19">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -213,6 +218,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -272,7 +292,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="116">
+  <x:cellXfs count="125">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -550,6 +570,21 @@
     <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1426,65 +1461,60 @@
       <x:c r="H11" s="105"/>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="114" t="str">
-        <x:v>MEASURED ENGINEERING RESULTS</x:v>
-      </x:c>
-      <x:c r="B13" s="114"/>
-      <x:c r="C13" s="114"/>
-      <x:c r="D13" s="114"/>
-      <x:c r="E13" s="114" t="str">
-        <x:v>ESTIMATED / MODELED OPPORTUNITIES</x:v>
-      </x:c>
-      <x:c r="F13" s="114"/>
-      <x:c r="G13" s="114"/>
-      <x:c r="H13" s="114"/>
+      <x:c r="A13" s="117" t="str">
+        <x:v>MODELED OPERATIONAL VALUE</x:v>
+      </x:c>
+      <x:c r="B13" s="117"/>
+      <x:c r="C13" s="117"/>
+      <x:c r="D13" s="117"/>
+      <x:c r="E13" s="117"/>
+      <x:c r="F13" s="117"/>
+      <x:c r="G13" s="117"/>
+      <x:c r="H13" s="117"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
-      <x:c r="A14" s="115" t="str">
-        <x:v>94.6% fewer replay-processing rows
-86.6% smaller local PostgreSQL fixture footprint</x:v>
-      </x:c>
-      <x:c r="B14" s="115"/>
-      <x:c r="C14" s="115"/>
-      <x:c r="D14" s="115"/>
-      <x:c r="E14" s="115" t="str">
-        <x:v>~90% retrieval-time reduction; ~87% storage-cost reduction; 30 hours/week and ~$52K annual labor value; up to 227.5K widgets/~$205K contribution-margin opportunity — all under documented assumptions</x:v>
-      </x:c>
-      <x:c r="F14" s="115"/>
-      <x:c r="G14" s="115"/>
-      <x:c r="H14" s="115"/>
+      <x:c r="A14" s="121" t="str">
+        <x:v>30 hours/week of reporting effort addressed (20 supervisor + 10 manager), representing about $52K in modeled annual labor value under documented assumptions.</x:v>
+      </x:c>
+      <x:c r="B14" s="121"/>
+      <x:c r="C14" s="121"/>
+      <x:c r="D14" s="121"/>
+      <x:c r="E14" s="121"/>
+      <x:c r="F14" s="121"/>
+      <x:c r="G14" s="121"/>
+      <x:c r="H14" s="121"/>
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="115"/>
-      <x:c r="B15" s="115"/>
-      <x:c r="C15" s="115"/>
-      <x:c r="D15" s="115"/>
-      <x:c r="E15" s="115"/>
-      <x:c r="F15" s="115"/>
-      <x:c r="G15" s="115"/>
-      <x:c r="H15" s="115"/>
+      <x:c r="A15" s="121"/>
+      <x:c r="B15" s="121"/>
+      <x:c r="C15" s="121"/>
+      <x:c r="D15" s="121"/>
+      <x:c r="E15" s="121"/>
+      <x:c r="F15" s="121"/>
+      <x:c r="G15" s="121"/>
+      <x:c r="H15" s="121"/>
     </x:row>
     <x:row r="16" ht="30" customHeight="1">
-      <x:c r="A16" s="115"/>
-      <x:c r="B16" s="115"/>
-      <x:c r="C16" s="115"/>
-      <x:c r="D16" s="115"/>
-      <x:c r="E16" s="115"/>
-      <x:c r="F16" s="115"/>
-      <x:c r="G16" s="115"/>
-      <x:c r="H16" s="115"/>
+      <x:c r="A16" s="121"/>
+      <x:c r="B16" s="121"/>
+      <x:c r="C16" s="121"/>
+      <x:c r="D16" s="121"/>
+      <x:c r="E16" s="121"/>
+      <x:c r="F16" s="121"/>
+      <x:c r="G16" s="121"/>
+      <x:c r="H16" s="121"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="111" t="str">
-        <x:v>Modeled figures are planning opportunities—not booked savings, realized margin, guaranteed outcomes, or blanket accuracy.</x:v>
-      </x:c>
-      <x:c r="B18" s="111"/>
-      <x:c r="C18" s="111"/>
-      <x:c r="D18" s="111"/>
-      <x:c r="E18" s="111"/>
-      <x:c r="F18" s="111"/>
-      <x:c r="G18" s="111"/>
-      <x:c r="H18" s="111"/>
+      <x:c r="A18" s="124" t="str">
+        <x:v>Planning opportunity—not booked savings, autonomous decisions, or a guaranteed outcome.</x:v>
+      </x:c>
+      <x:c r="B18" s="124"/>
+      <x:c r="C18" s="124"/>
+      <x:c r="D18" s="124"/>
+      <x:c r="E18" s="124"/>
+      <x:c r="F18" s="124"/>
+      <x:c r="G18" s="124"/>
+      <x:c r="H18" s="124"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1512,6 +1542,8 @@
     <x:mergeCell ref="A14:D16"/>
     <x:mergeCell ref="E14:H16"/>
     <x:mergeCell ref="A18:H18"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A14:H16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add operational intelligence and impact evidence
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Re1ba9bdb2f5842d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R55af15bb67c84264"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R92d81601b3df43d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R0e0bbcaf29f04b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R7244102fd84b4d3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rea4d9f1e0c4849be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intelligence Evidence" sheetId="4" r:id="R860b14727c434945"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="22">
+  <x:fonts count="24">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -142,8 +143,19 @@
       <x:color rgb="FF171717"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="21"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="13"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="19">
+  <x:fills count="23">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -233,6 +245,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -292,7 +324,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="125">
+  <x:cellXfs count="141">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -584,6 +616,34 @@
     <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1547,4 +1607,214 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>Operational intelligence — synthetic evidence and boundaries</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="127"/>
+      <x:c r="B2" s="127"/>
+      <x:c r="C2" s="127"/>
+      <x:c r="D2" s="127"/>
+      <x:c r="E2" s="127"/>
+      <x:c r="F2" s="127"/>
+      <x:c r="G2" s="127"/>
+      <x:c r="H2" s="127"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="129" t="str">
+        <x:v>Portfolio demonstration only — no production connection or autonomous decisions.</x:v>
+      </x:c>
+      <x:c r="B3" s="129"/>
+      <x:c r="C3" s="129"/>
+      <x:c r="D3" s="129"/>
+      <x:c r="E3" s="129"/>
+      <x:c r="F3" s="129"/>
+      <x:c r="G3" s="129"/>
+      <x:c r="H3" s="129"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="131" t="str">
+        <x:v>INTERFACE</x:v>
+      </x:c>
+      <x:c r="B5" s="131" t="str"/>
+      <x:c r="C5" s="131" t="str">
+        <x:v>CURRENT PURPOSE</x:v>
+      </x:c>
+      <x:c r="D5" s="131" t="str"/>
+      <x:c r="E5" s="131" t="str">
+        <x:v>VALIDATED BOUNDARY</x:v>
+      </x:c>
+      <x:c r="F5" s="131" t="str"/>
+      <x:c r="G5" s="131" t="str">
+        <x:v>VALUE SIGNAL</x:v>
+      </x:c>
+      <x:c r="H5" s="131" t="str"/>
+    </x:row>
+    <x:row r="6" ht="46" customHeight="1">
+      <x:c r="A6" s="135" t="str">
+        <x:v>Chatbot</x:v>
+      </x:c>
+      <x:c r="B6" s="135" t="str"/>
+      <x:c r="C6" s="135" t="str">
+        <x:v>Source-grounded report retrieval</x:v>
+      </x:c>
+      <x:c r="D6" s="135" t="str"/>
+      <x:c r="E6" s="135" t="str">
+        <x:v>Citations + deterministic fallback</x:v>
+      </x:c>
+      <x:c r="F6" s="135" t="str"/>
+      <x:c r="G6" s="135" t="str">
+        <x:v>Estimated ~90% faster retrieval</x:v>
+      </x:c>
+      <x:c r="H6" s="135" t="str"/>
+    </x:row>
+    <x:row r="7" ht="46" customHeight="1">
+      <x:c r="A7" s="135" t="str">
+        <x:v>Report doctor</x:v>
+      </x:c>
+      <x:c r="B7" s="135" t="str"/>
+      <x:c r="C7" s="135" t="str">
+        <x:v>Expected-output and exception diagnostics</x:v>
+      </x:c>
+      <x:c r="D7" s="135" t="str"/>
+      <x:c r="E7" s="135" t="str">
+        <x:v>Read-only; no repair or publication</x:v>
+      </x:c>
+      <x:c r="F7" s="135" t="str"/>
+      <x:c r="G7" s="135" t="str">
+        <x:v>Faster investigation</x:v>
+      </x:c>
+      <x:c r="H7" s="135" t="str"/>
+    </x:row>
+    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="A8" s="135" t="str">
+        <x:v>Governed oracle</x:v>
+      </x:c>
+      <x:c r="B8" s="135" t="str"/>
+      <x:c r="C8" s="135" t="str">
+        <x:v>Contract-bound interpretation and validation</x:v>
+      </x:c>
+      <x:c r="D8" s="135" t="str"/>
+      <x:c r="E8" s="135" t="str">
+        <x:v>Missing/ambiguous evidence fails closed</x:v>
+      </x:c>
+      <x:c r="F8" s="135" t="str"/>
+      <x:c r="G8" s="135" t="str">
+        <x:v>Consistent evidence checks</x:v>
+      </x:c>
+      <x:c r="H8" s="135" t="str"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="136" t="str">
+        <x:v>IMPACT METHODOLOGY</x:v>
+      </x:c>
+      <x:c r="B10" s="136"/>
+      <x:c r="C10" s="136"/>
+      <x:c r="D10" s="136"/>
+      <x:c r="E10" s="136"/>
+      <x:c r="F10" s="136"/>
+      <x:c r="G10" s="136"/>
+      <x:c r="H10" s="136"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11" s="139" t="str">
+        <x:v>Labor: 30 hours/week and about $52K modeled annual value. Retrieval: representative 20–30 minutes reduced to 1–2 minutes (~90% estimated). Downtime upper bound: 5 minutes × 1,000 widgets/hour/machine × 52.5 events/week × 52 weeks = up to 227,500 widgets; at $0.90/widget, approximately $205K modeled contribution-margin opportunity.</x:v>
+      </x:c>
+      <x:c r="B11" s="139"/>
+      <x:c r="C11" s="139"/>
+      <x:c r="D11" s="139"/>
+      <x:c r="E11" s="139"/>
+      <x:c r="F11" s="139"/>
+      <x:c r="G11" s="139"/>
+      <x:c r="H11" s="139"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12" s="139"/>
+      <x:c r="B12" s="139"/>
+      <x:c r="C12" s="139"/>
+      <x:c r="D12" s="139"/>
+      <x:c r="E12" s="139"/>
+      <x:c r="F12" s="139"/>
+      <x:c r="G12" s="139"/>
+      <x:c r="H12" s="139"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13" s="139"/>
+      <x:c r="B13" s="139"/>
+      <x:c r="C13" s="139"/>
+      <x:c r="D13" s="139"/>
+      <x:c r="E13" s="139"/>
+      <x:c r="F13" s="139"/>
+      <x:c r="G13" s="139"/>
+      <x:c r="H13" s="139"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14" s="139"/>
+      <x:c r="B14" s="139"/>
+      <x:c r="C14" s="139"/>
+      <x:c r="D14" s="139"/>
+      <x:c r="E14" s="139"/>
+      <x:c r="F14" s="139"/>
+      <x:c r="G14" s="139"/>
+      <x:c r="H14" s="139"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="140" t="str">
+        <x:v>Planning scenarios—not booked savings, realized production, guaranteed margin, or autonomous outcomes.</x:v>
+      </x:c>
+      <x:c r="B16" s="140"/>
+      <x:c r="C16" s="140"/>
+      <x:c r="D16" s="140"/>
+      <x:c r="E16" s="140"/>
+      <x:c r="F16" s="140"/>
+      <x:c r="G16" s="140"/>
+      <x:c r="H16" s="140"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="G7:H7"/>
+    <x:mergeCell ref="A8:B8"/>
+    <x:mergeCell ref="C8:D8"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="G8:H8"/>
+    <x:mergeCell ref="A10:H10"/>
+    <x:mergeCell ref="A11:H14"/>
+    <x:mergeCell ref="A16:H16"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Consolidate case study into progressive evidence paths
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,10 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R0e0bbcaf29f04b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R7244102fd84b4d3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rea4d9f1e0c4849be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intelligence Evidence" sheetId="4" r:id="R860b14727c434945"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4b0455644bc8472e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R0d5ad9a9b01f46aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R29eda74b27314fac"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intelligence Evidence" sheetId="4" r:id="R5b67e01bad8a4e87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="Re2126a2befbf44f6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R55ff62d0fab04a36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="Rbded34eb152345b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,10 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="$#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="24">
+  <x:fonts count="26">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -154,8 +161,20 @@
       <x:color rgb="FF171717"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF626262"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="23">
+  <x:fills count="27">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -267,8 +286,28 @@
         <x:fgColor rgb="FFF6F6F4"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -320,11 +359,25 @@
         <x:color rgb="FFD5DDD7"/>
       </x:top>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="141">
+  <x:cellXfs count="171">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -644,6 +697,66 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1729,71 +1842,67 @@
       </x:c>
       <x:c r="H8" s="135" t="str"/>
     </x:row>
-    <x:row r="10">
-      <x:c r="A10" s="136" t="str">
-        <x:v>IMPACT METHODOLOGY</x:v>
-      </x:c>
-      <x:c r="B10" s="136"/>
-      <x:c r="C10" s="136"/>
-      <x:c r="D10" s="136"/>
-      <x:c r="E10" s="136"/>
-      <x:c r="F10" s="136"/>
-      <x:c r="G10" s="136"/>
-      <x:c r="H10" s="136"/>
+    <x:row r="10" ht="32" customHeight="1">
+      <x:c r="A10" s="143" t="str">
+        <x:v>The interface sheet intentionally contains no impact calculations; those live once in Impact Model.</x:v>
+      </x:c>
+      <x:c r="B10" s="143"/>
+      <x:c r="C10" s="143"/>
+      <x:c r="D10" s="143"/>
+      <x:c r="E10" s="143"/>
+      <x:c r="F10" s="143"/>
+      <x:c r="G10" s="143"/>
+      <x:c r="H10" s="143"/>
     </x:row>
     <x:row r="11" ht="28" customHeight="1">
-      <x:c r="A11" s="139" t="str">
-        <x:v>Labor: 30 hours/week and about $52K modeled annual value. Retrieval: representative 20–30 minutes reduced to 1–2 minutes (~90% estimated). Downtime upper bound: 5 minutes × 1,000 widgets/hour/machine × 52.5 events/week × 52 weeks = up to 227,500 widgets; at $0.90/widget, approximately $205K modeled contribution-margin opportunity.</x:v>
-      </x:c>
-      <x:c r="B11" s="139"/>
-      <x:c r="C11" s="139"/>
-      <x:c r="D11" s="139"/>
-      <x:c r="E11" s="139"/>
-      <x:c r="F11" s="139"/>
-      <x:c r="G11" s="139"/>
-      <x:c r="H11" s="139"/>
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
     </x:row>
     <x:row r="12" ht="28" customHeight="1">
-      <x:c r="A12" s="139"/>
-      <x:c r="B12" s="139"/>
-      <x:c r="C12" s="139"/>
-      <x:c r="D12" s="139"/>
-      <x:c r="E12" s="139"/>
-      <x:c r="F12" s="139"/>
-      <x:c r="G12" s="139"/>
-      <x:c r="H12" s="139"/>
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
     </x:row>
     <x:row r="13" ht="28" customHeight="1">
-      <x:c r="A13" s="139"/>
-      <x:c r="B13" s="139"/>
-      <x:c r="C13" s="139"/>
-      <x:c r="D13" s="139"/>
-      <x:c r="E13" s="139"/>
-      <x:c r="F13" s="139"/>
-      <x:c r="G13" s="139"/>
-      <x:c r="H13" s="139"/>
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
     </x:row>
     <x:row r="14" ht="28" customHeight="1">
-      <x:c r="A14" s="139"/>
-      <x:c r="B14" s="139"/>
-      <x:c r="C14" s="139"/>
-      <x:c r="D14" s="139"/>
-      <x:c r="E14" s="139"/>
-      <x:c r="F14" s="139"/>
-      <x:c r="G14" s="139"/>
-      <x:c r="H14" s="139"/>
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="140" t="str">
-        <x:v>Planning scenarios—not booked savings, realized production, guaranteed margin, or autonomous outcomes.</x:v>
-      </x:c>
-      <x:c r="B16" s="140"/>
-      <x:c r="C16" s="140"/>
-      <x:c r="D16" s="140"/>
-      <x:c r="E16" s="140"/>
-      <x:c r="F16" s="140"/>
-      <x:c r="G16" s="140"/>
-      <x:c r="H16" s="140"/>
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1817,4 +1926,701 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Source lineage - synthetic trace</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>A compact inspection path from governed input to prepared output. No production identifiers.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="151" t="str">
+        <x:v>TRACE ID</x:v>
+      </x:c>
+      <x:c r="B5" s="151" t="str">
+        <x:v>SOURCE CATEGORY</x:v>
+      </x:c>
+      <x:c r="C5" s="151" t="str">
+        <x:v>SOURCE FACT</x:v>
+      </x:c>
+      <x:c r="D5" s="151" t="str">
+        <x:v>TRANSFORMATION</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="str">
+        <x:v>REPORT FIELD</x:v>
+      </x:c>
+      <x:c r="F5" s="151" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="G5" s="151" t="str">
+        <x:v>EVIDENCE STATE</x:v>
+      </x:c>
+      <x:c r="H5" s="151" t="str">
+        <x:v>REVIEW QUESTION</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="155" t="str">
+        <x:v>TR-001</x:v>
+      </x:c>
+      <x:c r="B6" s="155" t="str">
+        <x:v>Hourly production</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="str">
+        <x:v>1,240 good widgets</x:v>
+      </x:c>
+      <x:c r="D6" s="155" t="str">
+        <x:v>Normalize + reconcile</x:v>
+      </x:c>
+      <x:c r="E6" s="155" t="str">
+        <x:v>Good widgets</x:v>
+      </x:c>
+      <x:c r="F6" s="155" t="str">
+        <x:v>Daily Production</x:v>
+      </x:c>
+      <x:c r="G6" s="155" t="str">
+        <x:v>certified</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="str">
+        <x:v>Does the total conserve source rows?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="155" t="str">
+        <x:v>TR-002</x:v>
+      </x:c>
+      <x:c r="B7" s="155" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C7" s="155" t="str">
+        <x:v>12 rejected widgets</x:v>
+      </x:c>
+      <x:c r="D7" s="155" t="str">
+        <x:v>Preserve observed zero/missing semantics</x:v>
+      </x:c>
+      <x:c r="E7" s="155" t="str">
+        <x:v>Reject widgets</x:v>
+      </x:c>
+      <x:c r="F7" s="155" t="str">
+        <x:v>Daily Production</x:v>
+      </x:c>
+      <x:c r="G7" s="155" t="str">
+        <x:v>certified</x:v>
+      </x:c>
+      <x:c r="H7" s="155" t="str">
+        <x:v>Is missing evidence distinct from zero?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="155" t="str">
+        <x:v>TR-003</x:v>
+      </x:c>
+      <x:c r="B8" s="155" t="str">
+        <x:v>Machine event</x:v>
+      </x:c>
+      <x:c r="C8" s="155" t="str">
+        <x:v>18-minute downtime</x:v>
+      </x:c>
+      <x:c r="D8" s="155" t="str">
+        <x:v>Classify event + link machine</x:v>
+      </x:c>
+      <x:c r="E8" s="155" t="str">
+        <x:v>Downtime minutes</x:v>
+      </x:c>
+      <x:c r="F8" s="155" t="str">
+        <x:v>Weekly Downtime</x:v>
+      </x:c>
+      <x:c r="G8" s="155" t="str">
+        <x:v>read back</x:v>
+      </x:c>
+      <x:c r="H8" s="155" t="str">
+        <x:v>Does remote content match the candidate?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="155" t="str">
+        <x:v>TR-004</x:v>
+      </x:c>
+      <x:c r="B9" s="155" t="str">
+        <x:v>Labor note</x:v>
+      </x:c>
+      <x:c r="C9" s="155" t="str">
+        <x:v>Shift context entered</x:v>
+      </x:c>
+      <x:c r="D9" s="155" t="str">
+        <x:v>Attach source lineage</x:v>
+      </x:c>
+      <x:c r="E9" s="155" t="str">
+        <x:v>Supervisor context</x:v>
+      </x:c>
+      <x:c r="F9" s="155" t="str">
+        <x:v>Shift Draft</x:v>
+      </x:c>
+      <x:c r="G9" s="155" t="str">
+        <x:v>human review</x:v>
+      </x:c>
+      <x:c r="H9" s="155" t="str">
+        <x:v>What operational context must be added?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="157" t="str">
+        <x:v>Inspection rule: an output may advance only when identity, source lineage, semantics, publication state, and readback evidence agree.</x:v>
+      </x:c>
+      <x:c r="B11" s="157"/>
+      <x:c r="C11" s="157"/>
+      <x:c r="D11" s="157"/>
+      <x:c r="E11" s="157"/>
+      <x:c r="F11" s="157"/>
+      <x:c r="G11" s="157"/>
+      <x:c r="H11" s="157"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A11:H11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Exception review - synthetic operator cases</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>Examples show what the system surfaces and what remains a human decision.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="151" t="str">
+        <x:v>CASE</x:v>
+      </x:c>
+      <x:c r="B5" s="151" t="str">
+        <x:v>OBSERVED CONDITION</x:v>
+      </x:c>
+      <x:c r="C5" s="151" t="str">
+        <x:v>SYSTEM CLASSIFICATION</x:v>
+      </x:c>
+      <x:c r="D5" s="151" t="str">
+        <x:v>AUTOMATED BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="str">
+        <x:v>HUMAN REVIEW</x:v>
+      </x:c>
+      <x:c r="F5" s="151" t="str">
+        <x:v>WRITE AUTHORITY</x:v>
+      </x:c>
+      <x:c r="G5" s="151" t="str">
+        <x:v>SAFE OUTCOME</x:v>
+      </x:c>
+      <x:c r="H5" s="151" t="str">
+        <x:v>WHY IT MATTERS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="155" t="str">
+        <x:v>EX-01</x:v>
+      </x:c>
+      <x:c r="B6" s="155" t="str">
+        <x:v>Required source absent</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="str">
+        <x:v>pending_source</x:v>
+      </x:c>
+      <x:c r="D6" s="155" t="str">
+        <x:v>Retain expected output; do not publish</x:v>
+      </x:c>
+      <x:c r="E6" s="155" t="str">
+        <x:v>Confirm source arrival or operational exception</x:v>
+      </x:c>
+      <x:c r="F6" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G6" s="155" t="str">
+        <x:v>Missing remains missing</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="str">
+        <x:v>Prevents invented zeros</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="155" t="str">
+        <x:v>EX-02</x:v>
+      </x:c>
+      <x:c r="B7" s="155" t="str">
+        <x:v>Equivalent replay</x:v>
+      </x:c>
+      <x:c r="C7" s="155" t="str">
+        <x:v>exact_no_op</x:v>
+      </x:c>
+      <x:c r="D7" s="155" t="str">
+        <x:v>Compare governed material identity</x:v>
+      </x:c>
+      <x:c r="E7" s="155" t="str">
+        <x:v>No action unless context changed</x:v>
+      </x:c>
+      <x:c r="F7" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G7" s="155" t="str">
+        <x:v>Zero second write</x:v>
+      </x:c>
+      <x:c r="H7" s="155" t="str">
+        <x:v>Avoids duplicate versions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="155" t="str">
+        <x:v>EX-03</x:v>
+      </x:c>
+      <x:c r="B8" s="155" t="str">
+        <x:v>Write accepted; response lost</x:v>
+      </x:c>
+      <x:c r="C8" s="155" t="str">
+        <x:v>readback_pending</x:v>
+      </x:c>
+      <x:c r="D8" s="155" t="str">
+        <x:v>GET exact item; never repeat PUT</x:v>
+      </x:c>
+      <x:c r="E8" s="155" t="str">
+        <x:v>Review only if readback disagrees</x:v>
+      </x:c>
+      <x:c r="F8" s="155" t="str">
+        <x:v>GET only</x:v>
+      </x:c>
+      <x:c r="G8" s="155" t="str">
+        <x:v>Settle or fail closed</x:v>
+      </x:c>
+      <x:c r="H8" s="155" t="str">
+        <x:v>Bounds ambiguity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="155" t="str">
+        <x:v>EX-04</x:v>
+      </x:c>
+      <x:c r="B9" s="155" t="str">
+        <x:v>Contract or lineage drift</x:v>
+      </x:c>
+      <x:c r="C9" s="155" t="str">
+        <x:v>contract_refusal</x:v>
+      </x:c>
+      <x:c r="D9" s="155" t="str">
+        <x:v>Stop interpretation/publication</x:v>
+      </x:c>
+      <x:c r="E9" s="155" t="str">
+        <x:v>Investigate configuration or source change</x:v>
+      </x:c>
+      <x:c r="F9" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G9" s="155" t="str">
+        <x:v>Explicit refusal</x:v>
+      </x:c>
+      <x:c r="H9" s="155" t="str">
+        <x:v>Prevents silent semantic drift</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="159" t="str">
+        <x:v>Decision boundary: the platform prepares, classifies, and refuses. Supervisors and managers interpret context and choose operational action.</x:v>
+      </x:c>
+      <x:c r="B11" s="159"/>
+      <x:c r="C11" s="159"/>
+      <x:c r="D11" s="159"/>
+      <x:c r="E11" s="159"/>
+      <x:c r="F11" s="159"/>
+      <x:c r="G11" s="159"/>
+      <x:c r="H11" s="159"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A11:H11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Impact model - editable assumptions</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>Planning scenarios only. Inputs are editable; outputs are formulas, not booked results.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="150" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="B5" s="150" t="str">
+        <x:v>INPUT</x:v>
+      </x:c>
+      <x:c r="C5" s="150" t="str">
+        <x:v>VALUE</x:v>
+      </x:c>
+      <x:c r="D5" s="150" t="str">
+        <x:v>UNIT</x:v>
+      </x:c>
+      <x:c r="F5" s="156" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="G5" s="156" t="str">
+        <x:v>FORMULA</x:v>
+      </x:c>
+      <x:c r="H5" s="156" t="str">
+        <x:v>RESULT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B6" s="160" t="str">
+        <x:v>Supervisor hours/week</x:v>
+      </x:c>
+      <x:c r="C6" s="161" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D6" s="160" t="str">
+        <x:v>hours</x:v>
+      </x:c>
+      <x:c r="F6" s="163" t="str">
+        <x:v>Labor hours/year</x:v>
+      </x:c>
+      <x:c r="G6" s="169" t="str">
+        <x:v>(20 + 10) hours × 52 weeks</x:v>
+      </x:c>
+      <x:c r="H6" s="164" t="n">
+        <x:f>(C6+C7)*C8</x:f>
+        <x:v>1560</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B7" s="160" t="str">
+        <x:v>Manager hours/week</x:v>
+      </x:c>
+      <x:c r="C7" s="161" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D7" s="160" t="str">
+        <x:v>hours</x:v>
+      </x:c>
+      <x:c r="F7" s="163" t="str">
+        <x:v>Modeled labor value</x:v>
+      </x:c>
+      <x:c r="G7" s="169" t="str">
+        <x:v>Labor hours × $33.33/hour</x:v>
+      </x:c>
+      <x:c r="H7" s="165" t="n">
+        <x:f>H6*C9</x:f>
+        <x:v>51994.799999999996</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B8" s="160" t="str">
+        <x:v>Weeks/year</x:v>
+      </x:c>
+      <x:c r="C8" s="161" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D8" s="160" t="str">
+        <x:v>weeks</x:v>
+      </x:c>
+      <x:c r="F8" s="163" t="str">
+        <x:v>Estimated retrieval reduction</x:v>
+      </x:c>
+      <x:c r="G8" s="169" t="str">
+        <x:v>(25 minutes - 2 minutes) ÷ 25 minutes</x:v>
+      </x:c>
+      <x:c r="H8" s="166" t="n">
+        <x:f>(C10-C11)/C10</x:f>
+        <x:v>0.92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B9" s="160" t="str">
+        <x:v>Blended hourly value</x:v>
+      </x:c>
+      <x:c r="C9" s="161" t="n">
+        <x:v>33.33</x:v>
+      </x:c>
+      <x:c r="D9" s="160" t="str">
+        <x:v>$/hour</x:v>
+      </x:c>
+      <x:c r="F9" s="163" t="str">
+        <x:v>Widget opportunity</x:v>
+      </x:c>
+      <x:c r="G9" s="169" t="str">
+        <x:v>5 minutes ÷ 60 × 1,000 × 52.5 × 52</x:v>
+      </x:c>
+      <x:c r="H9" s="164" t="n">
+        <x:f>C12/60*C13*C14*C15</x:f>
+        <x:v>227500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="160" t="str">
+        <x:v>Retrieval</x:v>
+      </x:c>
+      <x:c r="B10" s="160" t="str">
+        <x:v>Baseline search</x:v>
+      </x:c>
+      <x:c r="C10" s="161" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D10" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="G10" s="170"/>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="160" t="str">
+        <x:v>Retrieval</x:v>
+      </x:c>
+      <x:c r="B11" s="160" t="str">
+        <x:v>Bounded retrieval</x:v>
+      </x:c>
+      <x:c r="C11" s="161" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="F11" s="157" t="str">
+        <x:v>Contribution-margin opportunity</x:v>
+      </x:c>
+      <x:c r="G11" s="99" t="str">
+        <x:v>Widget opportunity × $0.90/widget</x:v>
+      </x:c>
+      <x:c r="H11" s="167" t="n">
+        <x:f>H9*C16</x:f>
+        <x:v>204750</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B12" s="160" t="str">
+        <x:v>Response improvement</x:v>
+      </x:c>
+      <x:c r="C12" s="161" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D12" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B13" s="160" t="str">
+        <x:v>Throughput</x:v>
+      </x:c>
+      <x:c r="C13" s="161" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="D13" s="160" t="str">
+        <x:v>widgets/hour/machine</x:v>
+      </x:c>
+      <x:c r="F13" s="168" t="str">
+        <x:v>Limitations: representative time study, role-rate assumptions, event frequency, throughput, response improvement, and margin are scenario inputs. Outputs are not realized savings, guaranteed production, or autonomous outcomes.</x:v>
+      </x:c>
+      <x:c r="G13" s="168"/>
+      <x:c r="H13" s="168"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B14" s="160" t="str">
+        <x:v>Events/week</x:v>
+      </x:c>
+      <x:c r="C14" s="161" t="n">
+        <x:v>52.5</x:v>
+      </x:c>
+      <x:c r="D14" s="160" t="str">
+        <x:v>events</x:v>
+      </x:c>
+      <x:c r="F14" s="168"/>
+      <x:c r="G14" s="168"/>
+      <x:c r="H14" s="168"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B15" s="160" t="str">
+        <x:v>Weeks/year</x:v>
+      </x:c>
+      <x:c r="C15" s="161" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D15" s="160" t="str">
+        <x:v>weeks</x:v>
+      </x:c>
+      <x:c r="F15" s="168"/>
+      <x:c r="G15" s="168"/>
+      <x:c r="H15" s="168"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B16" s="160" t="str">
+        <x:v>Contribution margin</x:v>
+      </x:c>
+      <x:c r="C16" s="161" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D16" s="160" t="str">
+        <x:v>$/widget</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="F13:H15"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Clarify reporting assistant and viewer journey
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R4b0455644bc8472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R0d5ad9a9b01f46aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R29eda74b27314fac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Intelligence Evidence" sheetId="4" r:id="R5b67e01bad8a4e87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="Re2126a2befbf44f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R55ff62d0fab04a36"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="Rbded34eb152345b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R5b090524cf8b4709"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R4ac93ecf88a44435"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rcfde8f626a8347a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant Evidence" sheetId="4" r:id="R5bc288b0bd4b4370"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R66cef73d53644836"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R303657d5a4404f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R236ce13baa4648d4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1738,7 +1738,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="127" t="str">
-        <x:v>Operational intelligence — synthetic evidence and boundaries</x:v>
+        <x:v>Reporting Assistant — internal evidence and boundaries</x:v>
       </x:c>
       <x:c r="B1" s="127"/>
       <x:c r="C1" s="127"/>
@@ -1760,7 +1760,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="129" t="str">
-        <x:v>Portfolio demonstration only — no production connection or autonomous decisions.</x:v>
+        <x:v>One public assistant; three controlled internal subsystems. Synthetic evidence only — no production connection or autonomous decisions.</x:v>
       </x:c>
       <x:c r="B3" s="129"/>
       <x:c r="C3" s="129"/>
@@ -1772,7 +1772,7 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="131" t="str">
-        <x:v>INTERFACE</x:v>
+        <x:v>SUBSYSTEM</x:v>
       </x:c>
       <x:c r="B5" s="131" t="str"/>
       <x:c r="C5" s="131" t="str">
@@ -1844,7 +1844,7 @@
     </x:row>
     <x:row r="10" ht="32" customHeight="1">
       <x:c r="A10" s="143" t="str">
-        <x:v>The interface sheet intentionally contains no impact calculations; those live once in Impact Model.</x:v>
+        <x:v>Public materials present one Reporting Assistant; this technical sheet preserves internal subsystem names and boundaries.</x:v>
       </x:c>
       <x:c r="B10" s="143"/>
       <x:c r="C10" s="143"/>

</xml_diff>

<commit_message>
Preserve seven-sheet evidence workbook
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,9 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="Rc7244d06f81c465e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R56680de4911843d5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Evidence" sheetId="3" r:id="Rcea363d942cf4a34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R1758a175ab2e41aa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="Rbbea1f3cce644b42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R14e0e7c24f8540be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant Evidence" sheetId="4" r:id="R120125a1c8dc4dde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R7d5b502e136348fd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R7b615ea87e7742b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R9ef09e9c48944bc0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,10 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="1">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0"/>
+    <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
+    <x:numFmt numFmtId="202" formatCode="#,##0"/>
+    <x:numFmt numFmtId="203" formatCode="$#,##0"/>
+    <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="16">
+  <x:fonts count="27">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -32,7 +40,7 @@
     <x:font>
       <x:i/>
       <x:sz val="11"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -44,7 +52,7 @@
     <x:font>
       <x:b/>
       <x:sz val="22"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -55,13 +63,13 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFD52B1E"/>
+      <x:color rgb="FF155E4A"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -73,7 +81,7 @@
     <x:font>
       <x:i/>
       <x:sz val="11"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -89,7 +97,7 @@
     <x:font>
       <x:b/>
       <x:sz val="22"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -100,7 +108,13 @@
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="FF171717"/>
+      <x:color rgb="FF10201C"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF155E4A"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -109,13 +123,98 @@
       <x:color rgb="FFD52B1E"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="22"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FFD52B1E"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="14"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="21"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="13"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF626262"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF171717"/>
+      <x:name val="Aptos"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="30">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF10201C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9F99D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF155E4A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFDF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F1E7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF1D6"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -134,7 +233,77 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFFFFFFF"/>
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF6F6F4"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF171717"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -144,50 +313,79 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="FFEEEEEC"/>
+        <x:fgColor rgb="FF171717"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF4F4F2"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="9">
     <x:border/>
     <x:border>
       <x:left style="thin">
-        <x:color rgb="FFD0D0CD"/>
+        <x:color rgb="FFD5DDD7"/>
       </x:left>
       <x:top style="thin">
-        <x:color rgb="FFD0D0CD"/>
+        <x:color rgb="FFD5DDD7"/>
       </x:top>
     </x:border>
     <x:border>
       <x:right style="thin">
-        <x:color rgb="FFD0D0CD"/>
+        <x:color rgb="FFD5DDD7"/>
       </x:right>
       <x:top style="thin">
-        <x:color rgb="FFD0D0CD"/>
+        <x:color rgb="FFD5DDD7"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD5DDD7"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD5DDD7"/>
       </x:top>
     </x:border>
     <x:border>
       <x:left style="thin">
         <x:color rgb="FFD0D0CD"/>
       </x:left>
-      <x:bottom style="thin">
-        <x:color rgb="FFD0D0CD"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
       <x:right style="thin">
         <x:color rgb="FFD0D0CD"/>
       </x:right>
-      <x:bottom style="thin">
-        <x:color rgb="FFD0D0CD"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
-      <x:bottom style="thin">
-        <x:color rgb="FFD0D0CD"/>
-      </x:bottom>
-    </x:border>
-    <x:border>
       <x:top style="thin">
         <x:color rgb="FFD0D0CD"/>
       </x:top>
@@ -195,16 +393,11 @@
         <x:color rgb="FFD0D0CD"/>
       </x:bottom>
     </x:border>
-    <x:border>
-      <x:top style="thin">
-        <x:color rgb="FFD0D0CD"/>
-      </x:top>
-    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="77">
+  <x:cellXfs count="184">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -377,35 +570,253 @@
     <x:xf numFmtId="200" fontId="14" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="16" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="9" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="17" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="14" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="20" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="20" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="17" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="21" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="22" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="19" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="23" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="18" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="19" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="25" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="26" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="23" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="24" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="27" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="28" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0"/>
+    <x:xf numFmtId="0" fontId="26" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="26" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="26" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="2">
+  <x:dxfs count="1">
     <x:dxf>
       <x:font>
         <x:b/>
-        <x:color rgb="FFD52B1E"/>
+        <x:color rgb="FF155E4A"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFFBE8E6"/>
-        </x:patternFill>
-      </x:fill>
-    </x:dxf>
-    <x:dxf>
-      <x:fill>
-        <x:patternFill patternType="solid">
-          <x:bgColor rgb="FFF4F4F2"/>
+        <x:patternFill>
+          <x:bgColor rgb="FFDDF4E7"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -619,37 +1030,37 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="43" t="str">
+      <x:c r="A1" s="100" t="str">
         <x:v>Synthetic Reliability Report</x:v>
       </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-      <x:c r="G1" s="43"/>
+      <x:c r="B1" s="100"/>
+      <x:c r="C1" s="100"/>
+      <x:c r="D1" s="100"/>
+      <x:c r="E1" s="100"/>
+      <x:c r="F1" s="100"/>
+      <x:c r="G1" s="100"/>
       <x:c r="H1" s="43"/>
     </x:row>
     <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="43"/>
-      <x:c r="B2" s="43"/>
-      <x:c r="C2" s="43"/>
-      <x:c r="D2" s="43"/>
-      <x:c r="E2" s="43"/>
-      <x:c r="F2" s="43"/>
-      <x:c r="G2" s="43"/>
+      <x:c r="A2" s="100"/>
+      <x:c r="B2" s="100"/>
+      <x:c r="C2" s="100"/>
+      <x:c r="D2" s="100"/>
+      <x:c r="E2" s="100"/>
+      <x:c r="F2" s="100"/>
+      <x:c r="G2" s="100"/>
       <x:c r="H2" s="43"/>
     </x:row>
     <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="44" t="str">
+      <x:c r="A3" s="101" t="str">
         <x:v>Portfolio demonstration only - generalized architecture, synthetic values, no production connection</x:v>
       </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-      <x:c r="G3" s="44"/>
+      <x:c r="B3" s="101"/>
+      <x:c r="C3" s="101"/>
+      <x:c r="D3" s="101"/>
+      <x:c r="E3" s="101"/>
+      <x:c r="F3" s="101"/>
+      <x:c r="G3" s="101"/>
       <x:c r="H3" s="44"/>
     </x:row>
     <x:row r="4">
@@ -663,19 +1074,19 @@
       <x:c r="H4" s="45"/>
     </x:row>
     <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="46" t="str">
+      <x:c r="A5" s="102" t="str">
         <x:v>Total governed writes</x:v>
       </x:c>
-      <x:c r="B5" s="46" t="str"/>
-      <x:c r="C5" s="46" t="str">
+      <x:c r="B5" s="102" t="str"/>
+      <x:c r="C5" s="102" t="str">
         <x:v>Equivalent replay writes</x:v>
       </x:c>
-      <x:c r="D5" s="46" t="str"/>
-      <x:c r="E5" s="46" t="str">
+      <x:c r="D5" s="102" t="str"/>
+      <x:c r="E5" s="102" t="str">
         <x:v>Final remote version</x:v>
       </x:c>
-      <x:c r="F5" s="46" t="str"/>
-      <x:c r="G5" s="46" t="str">
+      <x:c r="F5" s="102" t="str"/>
+      <x:c r="G5" s="102" t="str">
         <x:v>Overlapping writers</x:v>
       </x:c>
       <x:c r="H5" s="46" t="str"/>
@@ -723,33 +1134,33 @@
       <x:c r="H8" s="45"/>
     </x:row>
     <x:row r="9" ht="28" customHeight="1">
-      <x:c r="A9" s="51" t="str">
+      <x:c r="A9" s="103" t="str">
         <x:v>Reliability controls demonstrated</x:v>
       </x:c>
-      <x:c r="B9" s="51"/>
-      <x:c r="C9" s="51"/>
-      <x:c r="D9" s="51"/>
-      <x:c r="E9" s="51"/>
-      <x:c r="F9" s="51"/>
-      <x:c r="G9" s="51"/>
+      <x:c r="B9" s="103"/>
+      <x:c r="C9" s="103"/>
+      <x:c r="D9" s="103"/>
+      <x:c r="E9" s="103"/>
+      <x:c r="F9" s="103"/>
+      <x:c r="G9" s="103"/>
       <x:c r="H9" s="51"/>
     </x:row>
     <x:row r="10" ht="28" customHeight="1">
-      <x:c r="A10" s="46" t="str">
+      <x:c r="A10" s="102" t="str">
         <x:v>Invariant</x:v>
       </x:c>
-      <x:c r="B10" s="46" t="str">
+      <x:c r="B10" s="102" t="str">
         <x:v>Mechanism</x:v>
       </x:c>
-      <x:c r="C10" s="46" t="str">
+      <x:c r="C10" s="102" t="str">
         <x:v>Synthetic result</x:v>
       </x:c>
-      <x:c r="D10" s="46" t="str">
+      <x:c r="D10" s="102" t="str">
         <x:v>Boundary</x:v>
       </x:c>
-      <x:c r="E10" s="46" t="str"/>
-      <x:c r="F10" s="46" t="str"/>
-      <x:c r="G10" s="46" t="str"/>
+      <x:c r="E10" s="102" t="str"/>
+      <x:c r="F10" s="102" t="str"/>
+      <x:c r="G10" s="102" t="str"/>
       <x:c r="H10" s="46" t="str"/>
     </x:row>
     <x:row r="11" ht="44" customHeight="1">
@@ -759,7 +1170,7 @@
       <x:c r="B11" s="52" t="str">
         <x:v>Governed material identity</x:v>
       </x:c>
-      <x:c r="C11" s="53" t="str">
+      <x:c r="C11" s="78" t="str">
         <x:v>Exact no-op / zero writes</x:v>
       </x:c>
       <x:c r="D11" s="52" t="str">
@@ -777,7 +1188,7 @@
       <x:c r="B12" s="54" t="str">
         <x:v>Retained candidate plus GET</x:v>
       </x:c>
-      <x:c r="C12" s="55" t="str">
+      <x:c r="C12" s="79" t="str">
         <x:v>Settled / zero retry writes</x:v>
       </x:c>
       <x:c r="D12" s="54" t="str">
@@ -795,7 +1206,7 @@
       <x:c r="B13" s="52" t="str">
         <x:v>Durable expected output</x:v>
       </x:c>
-      <x:c r="C13" s="53" t="str">
+      <x:c r="C13" s="78" t="str">
         <x:v>Same item advanced once</x:v>
       </x:c>
       <x:c r="D13" s="52" t="str">
@@ -813,7 +1224,7 @@
       <x:c r="B14" s="54" t="str">
         <x:v>Exclusive writer lease</x:v>
       </x:c>
-      <x:c r="C14" s="55" t="str">
+      <x:c r="C14" s="79" t="str">
         <x:v>Second writer refused</x:v>
       </x:c>
       <x:c r="D14" s="54" t="str">
@@ -831,7 +1242,7 @@
       <x:c r="B15" s="52" t="str">
         <x:v>Immutable prior release</x:v>
       </x:c>
-      <x:c r="C15" s="53" t="str">
+      <x:c r="C15" s="78" t="str">
         <x:v>Exact rollback restored</x:v>
       </x:c>
       <x:c r="D15" s="52" t="str">
@@ -853,15 +1264,15 @@
       <x:c r="H16" s="45"/>
     </x:row>
     <x:row r="17" ht="42" customHeight="1">
-      <x:c r="A17" s="56" t="str">
+      <x:c r="A17" s="104" t="str">
         <x:v>Claim boundary: this workbook demonstrates reliability behavior only; it does not represent production data, financial impact, or blanket accuracy.</x:v>
       </x:c>
-      <x:c r="B17" s="56"/>
-      <x:c r="C17" s="56"/>
-      <x:c r="D17" s="56"/>
-      <x:c r="E17" s="56"/>
-      <x:c r="F17" s="56"/>
-      <x:c r="G17" s="56"/>
+      <x:c r="B17" s="104"/>
+      <x:c r="C17" s="104"/>
+      <x:c r="D17" s="104"/>
+      <x:c r="E17" s="104"/>
+      <x:c r="F17" s="104"/>
+      <x:c r="G17" s="104"/>
       <x:c r="H17" s="56"/>
     </x:row>
   </x:sheetData>
@@ -905,31 +1316,31 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="59" t="str">
+      <x:c r="A1" s="105" t="str">
         <x:v>Step</x:v>
       </x:c>
-      <x:c r="B1" s="59" t="str">
+      <x:c r="B1" s="105" t="str">
         <x:v>Event</x:v>
       </x:c>
-      <x:c r="C1" s="59" t="str">
+      <x:c r="C1" s="105" t="str">
         <x:v>State</x:v>
       </x:c>
-      <x:c r="D1" s="59" t="str">
+      <x:c r="D1" s="105" t="str">
         <x:v>Material</x:v>
       </x:c>
-      <x:c r="E1" s="59" t="str">
+      <x:c r="E1" s="105" t="str">
         <x:v>Remote version</x:v>
       </x:c>
-      <x:c r="F1" s="59" t="str">
+      <x:c r="F1" s="105" t="str">
         <x:v>Writes</x:v>
       </x:c>
-      <x:c r="G1" s="59" t="str">
+      <x:c r="G1" s="105" t="str">
         <x:v>Settlement</x:v>
       </x:c>
-      <x:c r="H1" s="59" t="str">
+      <x:c r="H1" s="105" t="str">
         <x:v>Result</x:v>
       </x:c>
-      <x:c r="I1" s="59" t="str">
+      <x:c r="I1" s="105" t="str">
         <x:v>Writer overlap</x:v>
       </x:c>
     </x:row>
@@ -992,31 +1403,31 @@
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="72" t="n">
+      <x:c r="A4" s="108" t="n">
         <x:v>3</x:v>
       </x:c>
-      <x:c r="B4" s="68" t="str">
+      <x:c r="B4" s="109" t="str">
         <x:v>Equivalent capture marker changes</x:v>
       </x:c>
-      <x:c r="C4" s="68" t="str">
+      <x:c r="C4" s="109" t="str">
         <x:v>certified</x:v>
       </x:c>
-      <x:c r="D4" s="68" t="str">
+      <x:c r="D4" s="109" t="str">
         <x:v>material-a</x:v>
       </x:c>
-      <x:c r="E4" s="72" t="n">
+      <x:c r="E4" s="108" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F4" s="72" t="n">
+      <x:c r="F4" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G4" s="68" t="str">
+      <x:c r="G4" s="109" t="str">
         <x:v>exact GET</x:v>
       </x:c>
-      <x:c r="H4" s="68" t="str">
+      <x:c r="H4" s="109" t="str">
         <x:v>exact no-op</x:v>
       </x:c>
-      <x:c r="I4" s="72" t="n">
+      <x:c r="I4" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1050,31 +1461,31 @@
       </x:c>
     </x:row>
     <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="72" t="n">
+      <x:c r="A6" s="108" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="B6" s="68" t="str">
+      <x:c r="B6" s="109" t="str">
         <x:v>Equivalent replay after settlement</x:v>
       </x:c>
-      <x:c r="C6" s="68" t="str">
+      <x:c r="C6" s="109" t="str">
         <x:v>certified</x:v>
       </x:c>
-      <x:c r="D6" s="68" t="str">
+      <x:c r="D6" s="109" t="str">
         <x:v>material-b</x:v>
       </x:c>
-      <x:c r="E6" s="72" t="n">
+      <x:c r="E6" s="108" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="F6" s="72" t="n">
+      <x:c r="F6" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G6" s="68" t="str">
+      <x:c r="G6" s="109" t="str">
         <x:v>exact GET</x:v>
       </x:c>
-      <x:c r="H6" s="68" t="str">
+      <x:c r="H6" s="109" t="str">
         <x:v>exact no-op</x:v>
       </x:c>
-      <x:c r="I6" s="72" t="n">
+      <x:c r="I6" s="108" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1121,160 +1532,1205 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="20" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="42" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="31" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="40" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="34" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="19" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="26" customHeight="1">
-      <x:c r="A1" s="43" t="str">
-        <x:v>Impact Evidence Guide</x:v>
-      </x:c>
-      <x:c r="B1" s="43"/>
-      <x:c r="C1" s="43"/>
-      <x:c r="D1" s="43"/>
-      <x:c r="E1" s="43"/>
-      <x:c r="F1" s="43"/>
-    </x:row>
-    <x:row r="2" ht="26" customHeight="1">
-      <x:c r="A2" s="43"/>
-      <x:c r="B2" s="43"/>
-      <x:c r="C2" s="43"/>
-      <x:c r="D2" s="43"/>
-      <x:c r="E2" s="43"/>
-      <x:c r="F2" s="43"/>
-    </x:row>
-    <x:row r="3" ht="28" customHeight="1">
-      <x:c r="A3" s="44" t="str">
-        <x:v>Documented observations and planning models - no production records included</x:v>
-      </x:c>
-      <x:c r="B3" s="44"/>
-      <x:c r="C3" s="44"/>
-      <x:c r="D3" s="44"/>
-      <x:c r="E3" s="44"/>
-      <x:c r="F3" s="44"/>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="45"/>
-      <x:c r="B4" s="45"/>
-      <x:c r="C4" s="45"/>
-      <x:c r="D4" s="45"/>
-      <x:c r="E4" s="45"/>
-      <x:c r="F4" s="45"/>
-    </x:row>
-    <x:row r="5" ht="34" customHeight="1">
-      <x:c r="A5" s="76" t="str">
-        <x:v>Evidence</x:v>
-      </x:c>
-      <x:c r="B5" s="76" t="str">
-        <x:v>Class</x:v>
-      </x:c>
-      <x:c r="C5" s="76" t="str">
-        <x:v>Basis</x:v>
-      </x:c>
-      <x:c r="D5" s="76" t="str">
-        <x:v>Result</x:v>
-      </x:c>
-      <x:c r="E5" s="76" t="str">
-        <x:v>Interpretation</x:v>
-      </x:c>
-      <x:c r="F5" s="76" t="str">
-        <x:v>Limit</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="58" customHeight="1">
-      <x:c r="A6" s="67" t="str">
-        <x:v>Production-count schema</x:v>
-      </x:c>
-      <x:c r="B6" s="67" t="str">
-        <x:v>Reviewed observation</x:v>
-      </x:c>
-      <x:c r="C6" s="67" t="str">
-        <x:v>Approximately six months; about one in four legacy reports did not conform</x:v>
-      </x:c>
-      <x:c r="D6" s="67" t="str">
-        <x:v>About 75% → 100%</x:v>
-      </x:c>
-      <x:c r="E6" s="67" t="str">
-        <x:v>25 percentage-point increase across reviewed system outputs</x:v>
-      </x:c>
-      <x:c r="F6" s="67" t="str">
-        <x:v>Sample-bound; exact N/date range retained privately</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="58" customHeight="1">
-      <x:c r="A7" s="68" t="str">
-        <x:v>Reporting effort</x:v>
-      </x:c>
-      <x:c r="B7" s="68" t="str">
-        <x:v>Modeled</x:v>
-      </x:c>
-      <x:c r="C7" s="68" t="str">
-        <x:v>20 supervisor + 10 manager hours/week</x:v>
-      </x:c>
-      <x:c r="D7" s="68" t="str">
-        <x:v>30 hours/week · about $52K/year</x:v>
-      </x:c>
-      <x:c r="E7" s="68" t="str">
-        <x:v>Potential time redirected from preparation to review</x:v>
-      </x:c>
-      <x:c r="F7" s="68" t="str">
-        <x:v>Not booked savings</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="58" customHeight="1">
-      <x:c r="A8" s="68" t="str">
-        <x:v>Report retrieval</x:v>
-      </x:c>
-      <x:c r="B8" s="68" t="str">
-        <x:v>Estimated</x:v>
-      </x:c>
-      <x:c r="C8" s="68" t="str">
-        <x:v>Representative 20-30 minute search reduced to 1-2 minutes</x:v>
-      </x:c>
-      <x:c r="D8" s="68" t="str">
-        <x:v>About 90% faster</x:v>
-      </x:c>
-      <x:c r="E8" s="68" t="str">
-        <x:v>Faster access to cited evidence</x:v>
-      </x:c>
-      <x:c r="F8" s="68" t="str">
-        <x:v>Scenario-dependent</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9" ht="58" customHeight="1">
-      <x:c r="A9" s="69" t="str">
-        <x:v>Downtime response</x:v>
-      </x:c>
-      <x:c r="B9" s="69" t="str">
-        <x:v>Modeled upper bound</x:v>
-      </x:c>
-      <x:c r="C9" s="69" t="str">
-        <x:v>5 minutes × 1,000 production units/hour/machine × 52.5 events/week × 52 weeks</x:v>
-      </x:c>
-      <x:c r="D9" s="69" t="str">
-        <x:v>Up to 227,500 production units · about $205K</x:v>
-      </x:c>
-      <x:c r="E9" s="69" t="str">
-        <x:v>Sensitivity model for prioritization</x:v>
-      </x:c>
-      <x:c r="F9" s="69" t="str">
-        <x:v>Not realized production or margin</x:v>
-      </x:c>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="110" t="str">
+        <x:v>Prepared outputs for human review and action</x:v>
+      </x:c>
+      <x:c r="B1" s="110"/>
+      <x:c r="C1" s="110"/>
+      <x:c r="D1" s="110"/>
+      <x:c r="E1" s="110"/>
+      <x:c r="F1" s="110"/>
+      <x:c r="G1" s="110"/>
+      <x:c r="H1" s="110"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="110"/>
+      <x:c r="B2" s="110"/>
+      <x:c r="C2" s="110"/>
+      <x:c r="D2" s="110"/>
+      <x:c r="E2" s="110"/>
+      <x:c r="F2" s="110"/>
+      <x:c r="G2" s="110"/>
+      <x:c r="H2" s="110"/>
+    </x:row>
+    <x:row r="3" ht="30" customHeight="1">
+      <x:c r="A3" s="111" t="str">
+        <x:v>Synthetic portfolio guide — no production connection; the platform supports decisions and does not make them.</x:v>
+      </x:c>
+      <x:c r="B3" s="111"/>
+      <x:c r="C3" s="111"/>
+      <x:c r="D3" s="111"/>
+      <x:c r="E3" s="111"/>
+      <x:c r="F3" s="111"/>
+      <x:c r="G3" s="111"/>
+      <x:c r="H3" s="111"/>
+    </x:row>
+    <x:row r="5" ht="24" customHeight="1">
+      <x:c r="A5" s="112" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="B5" s="112" t="str"/>
+      <x:c r="C5" s="112" t="str">
+        <x:v>PRIMARY USER</x:v>
+      </x:c>
+      <x:c r="D5" s="112" t="str"/>
+      <x:c r="E5" s="112" t="str">
+        <x:v>WHAT AUTOMATION PREPARES</x:v>
+      </x:c>
+      <x:c r="F5" s="112" t="str"/>
+      <x:c r="G5" s="112" t="str">
+        <x:v>HUMAN USE</x:v>
+      </x:c>
+      <x:c r="H5" s="112" t="str"/>
+    </x:row>
+    <x:row r="6" ht="48" customHeight="1">
+      <x:c r="A6" s="113" t="str">
+        <x:v>Shift Drafts</x:v>
+      </x:c>
+      <x:c r="B6" s="113" t="str"/>
+      <x:c r="C6" s="113" t="str">
+        <x:v>Supervisors</x:v>
+      </x:c>
+      <x:c r="D6" s="113" t="str"/>
+      <x:c r="E6" s="113" t="str">
+        <x:v>Collection, reconciliation, organization, spreadsheet preparation</x:v>
+      </x:c>
+      <x:c r="F6" s="113" t="str"/>
+      <x:c r="G6" s="113" t="str">
+        <x:v>Review exceptions, add context, finalize</x:v>
+      </x:c>
+      <x:c r="H6" s="113" t="str"/>
+    </x:row>
+    <x:row r="7" ht="48" customHeight="1">
+      <x:c r="A7" s="113" t="str">
+        <x:v>Daily Production Reports</x:v>
+      </x:c>
+      <x:c r="B7" s="113" t="str"/>
+      <x:c r="C7" s="113" t="str">
+        <x:v>Managers</x:v>
+      </x:c>
+      <x:c r="D7" s="113" t="str"/>
+      <x:c r="E7" s="113" t="str">
+        <x:v>Production, molding, labor, quality, plan attainment, downtime</x:v>
+      </x:c>
+      <x:c r="F7" s="113" t="str"/>
+      <x:c r="G7" s="113" t="str">
+        <x:v>Investigate constraints; prioritize staffing, plan, maintenance, or coordination follow-up</x:v>
+      </x:c>
+      <x:c r="H7" s="113" t="str"/>
+    </x:row>
+    <x:row r="8" ht="48" customHeight="1">
+      <x:c r="A8" s="113" t="str">
+        <x:v>Weekly Production Reports</x:v>
+      </x:c>
+      <x:c r="B8" s="113" t="str"/>
+      <x:c r="C8" s="113" t="str">
+        <x:v>Managers / teams</x:v>
+      </x:c>
+      <x:c r="D8" s="113" t="str"/>
+      <x:c r="E8" s="113" t="str">
+        <x:v>Comparable period views and source-linked trends</x:v>
+      </x:c>
+      <x:c r="F8" s="113" t="str"/>
+      <x:c r="G8" s="113" t="str">
+        <x:v>Capacity and labor planning; process improvement; weekly reviews</x:v>
+      </x:c>
+      <x:c r="H8" s="113" t="str"/>
+    </x:row>
+    <x:row r="9" ht="48" customHeight="1">
+      <x:c r="A9" s="113" t="str">
+        <x:v>Weekly Downtime Reports</x:v>
+      </x:c>
+      <x:c r="B9" s="113" t="str"/>
+      <x:c r="C9" s="113" t="str">
+        <x:v>Managers / maintenance</x:v>
+      </x:c>
+      <x:c r="D9" s="113" t="str"/>
+      <x:c r="E9" s="113" t="str">
+        <x:v>Recurring-versus-isolated event patterns and downtime evidence</x:v>
+      </x:c>
+      <x:c r="F9" s="113" t="str"/>
+      <x:c r="G9" s="113" t="str">
+        <x:v>Maintenance prioritization; meetings; shift handoffs</x:v>
+      </x:c>
+      <x:c r="H9" s="113" t="str"/>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="105" t="str">
+        <x:v>Operational input → ingestion → reconciliation and source linkage → validation → prepared output → human review → operational action</x:v>
+      </x:c>
+      <x:c r="B11" s="105"/>
+      <x:c r="C11" s="105"/>
+      <x:c r="D11" s="105"/>
+      <x:c r="E11" s="105"/>
+      <x:c r="F11" s="105"/>
+      <x:c r="G11" s="105"/>
+      <x:c r="H11" s="105"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="117" t="str">
+        <x:v>MODELED OPERATIONAL VALUE</x:v>
+      </x:c>
+      <x:c r="B13" s="117"/>
+      <x:c r="C13" s="117"/>
+      <x:c r="D13" s="117"/>
+      <x:c r="E13" s="117"/>
+      <x:c r="F13" s="117"/>
+      <x:c r="G13" s="117"/>
+      <x:c r="H13" s="117"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="121" t="str">
+        <x:v>30 hours/week of reporting effort addressed (20 supervisor + 10 manager), representing about $52K in modeled annual labor value under documented assumptions.</x:v>
+      </x:c>
+      <x:c r="B14" s="121"/>
+      <x:c r="C14" s="121"/>
+      <x:c r="D14" s="121"/>
+      <x:c r="E14" s="121"/>
+      <x:c r="F14" s="121"/>
+      <x:c r="G14" s="121"/>
+      <x:c r="H14" s="121"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="121"/>
+      <x:c r="B15" s="121"/>
+      <x:c r="C15" s="121"/>
+      <x:c r="D15" s="121"/>
+      <x:c r="E15" s="121"/>
+      <x:c r="F15" s="121"/>
+      <x:c r="G15" s="121"/>
+      <x:c r="H15" s="121"/>
+    </x:row>
+    <x:row r="16" ht="30" customHeight="1">
+      <x:c r="A16" s="121"/>
+      <x:c r="B16" s="121"/>
+      <x:c r="C16" s="121"/>
+      <x:c r="D16" s="121"/>
+      <x:c r="E16" s="121"/>
+      <x:c r="F16" s="121"/>
+      <x:c r="G16" s="121"/>
+      <x:c r="H16" s="121"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="124" t="str">
+        <x:v>Planning opportunity—not booked savings, autonomous decisions, or a guaranteed outcome.</x:v>
+      </x:c>
+      <x:c r="B18" s="124"/>
+      <x:c r="C18" s="124"/>
+      <x:c r="D18" s="124"/>
+      <x:c r="E18" s="124"/>
+      <x:c r="F18" s="124"/>
+      <x:c r="G18" s="124"/>
+      <x:c r="H18" s="124"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:F2"/>
-    <x:mergeCell ref="A3:F3"/>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="G7:H7"/>
+    <x:mergeCell ref="A8:B8"/>
+    <x:mergeCell ref="C8:D8"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="G8:H8"/>
+    <x:mergeCell ref="A9:B9"/>
+    <x:mergeCell ref="C9:D9"/>
+    <x:mergeCell ref="E9:F9"/>
+    <x:mergeCell ref="G9:H9"/>
+    <x:mergeCell ref="A11:H11"/>
+    <x:mergeCell ref="A13:D13"/>
+    <x:mergeCell ref="E13:H13"/>
+    <x:mergeCell ref="A14:D16"/>
+    <x:mergeCell ref="E14:H16"/>
+    <x:mergeCell ref="A18:H18"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A14:H16"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="A6:F9">
-    <x:cfRule type="expression" dxfId="1" priority="1">
-      <x:formula>MOD(ROW(),2)=0</x:formula>
-    </x:cfRule>
-  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="127" t="str">
+        <x:v>Reporting Assistant — internal evidence and boundaries</x:v>
+      </x:c>
+      <x:c r="B1" s="127"/>
+      <x:c r="C1" s="127"/>
+      <x:c r="D1" s="127"/>
+      <x:c r="E1" s="127"/>
+      <x:c r="F1" s="127"/>
+      <x:c r="G1" s="127"/>
+      <x:c r="H1" s="127"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="127"/>
+      <x:c r="B2" s="127"/>
+      <x:c r="C2" s="127"/>
+      <x:c r="D2" s="127"/>
+      <x:c r="E2" s="127"/>
+      <x:c r="F2" s="127"/>
+      <x:c r="G2" s="127"/>
+      <x:c r="H2" s="127"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="129" t="str">
+        <x:v>One public assistant; three controlled internal subsystems. Synthetic evidence only — no production connection or autonomous decisions.</x:v>
+      </x:c>
+      <x:c r="B3" s="129"/>
+      <x:c r="C3" s="129"/>
+      <x:c r="D3" s="129"/>
+      <x:c r="E3" s="129"/>
+      <x:c r="F3" s="129"/>
+      <x:c r="G3" s="129"/>
+      <x:c r="H3" s="129"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="131" t="str">
+        <x:v>SUBSYSTEM</x:v>
+      </x:c>
+      <x:c r="B5" s="131" t="str"/>
+      <x:c r="C5" s="131" t="str">
+        <x:v>CURRENT PURPOSE</x:v>
+      </x:c>
+      <x:c r="D5" s="131" t="str"/>
+      <x:c r="E5" s="131" t="str">
+        <x:v>VALIDATED BOUNDARY</x:v>
+      </x:c>
+      <x:c r="F5" s="131" t="str"/>
+      <x:c r="G5" s="131" t="str">
+        <x:v>VALUE SIGNAL</x:v>
+      </x:c>
+      <x:c r="H5" s="131" t="str"/>
+    </x:row>
+    <x:row r="6" ht="46" customHeight="1">
+      <x:c r="A6" s="135" t="str">
+        <x:v>Chatbot</x:v>
+      </x:c>
+      <x:c r="B6" s="135" t="str"/>
+      <x:c r="C6" s="135" t="str">
+        <x:v>Source-grounded report retrieval</x:v>
+      </x:c>
+      <x:c r="D6" s="135" t="str"/>
+      <x:c r="E6" s="135" t="str">
+        <x:v>Citations + deterministic fallback</x:v>
+      </x:c>
+      <x:c r="F6" s="135" t="str"/>
+      <x:c r="G6" s="135" t="str">
+        <x:v>Estimated ~90% faster retrieval</x:v>
+      </x:c>
+      <x:c r="H6" s="135" t="str"/>
+    </x:row>
+    <x:row r="7" ht="46" customHeight="1">
+      <x:c r="A7" s="135" t="str">
+        <x:v>Report doctor</x:v>
+      </x:c>
+      <x:c r="B7" s="135" t="str"/>
+      <x:c r="C7" s="135" t="str">
+        <x:v>Expected-output and exception diagnostics</x:v>
+      </x:c>
+      <x:c r="D7" s="135" t="str"/>
+      <x:c r="E7" s="135" t="str">
+        <x:v>Read-only; no repair or publication</x:v>
+      </x:c>
+      <x:c r="F7" s="135" t="str"/>
+      <x:c r="G7" s="135" t="str">
+        <x:v>Faster investigation</x:v>
+      </x:c>
+      <x:c r="H7" s="135" t="str"/>
+    </x:row>
+    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="A8" s="135" t="str">
+        <x:v>Governed oracle</x:v>
+      </x:c>
+      <x:c r="B8" s="135" t="str"/>
+      <x:c r="C8" s="135" t="str">
+        <x:v>Contract-bound interpretation and validation</x:v>
+      </x:c>
+      <x:c r="D8" s="135" t="str"/>
+      <x:c r="E8" s="135" t="str">
+        <x:v>Missing/ambiguous evidence fails closed</x:v>
+      </x:c>
+      <x:c r="F8" s="135" t="str"/>
+      <x:c r="G8" s="135" t="str">
+        <x:v>Consistent evidence checks</x:v>
+      </x:c>
+      <x:c r="H8" s="135" t="str"/>
+    </x:row>
+    <x:row r="10" ht="32" customHeight="1">
+      <x:c r="A10" s="143" t="str">
+        <x:v>Public materials present one Reporting Assistant; this technical sheet preserves internal subsystem names and boundaries.</x:v>
+      </x:c>
+      <x:c r="B10" s="143"/>
+      <x:c r="C10" s="143"/>
+      <x:c r="D10" s="143"/>
+      <x:c r="E10" s="143"/>
+      <x:c r="F10" s="143"/>
+      <x:c r="G10" s="143"/>
+      <x:c r="H10" s="143"/>
+    </x:row>
+    <x:row r="11" ht="28" customHeight="1">
+      <x:c r="A11"/>
+      <x:c r="B11"/>
+      <x:c r="C11"/>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
+    </x:row>
+    <x:row r="12" ht="28" customHeight="1">
+      <x:c r="A12"/>
+      <x:c r="B12"/>
+      <x:c r="C12"/>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
+    </x:row>
+    <x:row r="13" ht="28" customHeight="1">
+      <x:c r="A13"/>
+      <x:c r="B13"/>
+      <x:c r="C13"/>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
+    </x:row>
+    <x:row r="14" ht="28" customHeight="1">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A6:B6"/>
+    <x:mergeCell ref="C6:D6"/>
+    <x:mergeCell ref="E6:F6"/>
+    <x:mergeCell ref="G6:H6"/>
+    <x:mergeCell ref="A7:B7"/>
+    <x:mergeCell ref="C7:D7"/>
+    <x:mergeCell ref="E7:F7"/>
+    <x:mergeCell ref="G7:H7"/>
+    <x:mergeCell ref="A8:B8"/>
+    <x:mergeCell ref="C8:D8"/>
+    <x:mergeCell ref="E8:F8"/>
+    <x:mergeCell ref="G8:H8"/>
+    <x:mergeCell ref="A10:H10"/>
+    <x:mergeCell ref="A11:H14"/>
+    <x:mergeCell ref="A16:H16"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Source lineage - synthetic trace</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>A compact inspection path from governed input to prepared output. No production identifiers.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5" ht="36" customHeight="1">
+      <x:c r="A5" s="151" t="str">
+        <x:v>TRACE ID</x:v>
+      </x:c>
+      <x:c r="B5" s="151" t="str">
+        <x:v>SOURCE CATEGORY</x:v>
+      </x:c>
+      <x:c r="C5" s="151" t="str">
+        <x:v>SOURCE FACT</x:v>
+      </x:c>
+      <x:c r="D5" s="151" t="str">
+        <x:v>TRANSFORMATION</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="str">
+        <x:v>REPORT FIELD</x:v>
+      </x:c>
+      <x:c r="F5" s="151" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="G5" s="151" t="str">
+        <x:v>EVIDENCE STATE</x:v>
+      </x:c>
+      <x:c r="H5" s="151" t="str">
+        <x:v>REVIEW QUESTION</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="56" customHeight="1">
+      <x:c r="A6" s="155" t="str">
+        <x:v>TR-001</x:v>
+      </x:c>
+      <x:c r="B6" s="155" t="str">
+        <x:v>Hourly production</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="str">
+        <x:v>1,240 good production units</x:v>
+      </x:c>
+      <x:c r="D6" s="155" t="str">
+        <x:v>Normalize + reconcile</x:v>
+      </x:c>
+      <x:c r="E6" s="155" t="str">
+        <x:v>Good production units</x:v>
+      </x:c>
+      <x:c r="F6" s="155" t="str">
+        <x:v>Daily Production</x:v>
+      </x:c>
+      <x:c r="G6" s="155" t="str">
+        <x:v>certified</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="str">
+        <x:v>Does the total conserve source rows?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="56" customHeight="1">
+      <x:c r="A7" s="155" t="str">
+        <x:v>TR-002</x:v>
+      </x:c>
+      <x:c r="B7" s="155" t="str">
+        <x:v>Quality</x:v>
+      </x:c>
+      <x:c r="C7" s="155" t="str">
+        <x:v>12 rejected production units</x:v>
+      </x:c>
+      <x:c r="D7" s="155" t="str">
+        <x:v>Preserve observed zero/missing semantics</x:v>
+      </x:c>
+      <x:c r="E7" s="155" t="str">
+        <x:v>Rejected production units</x:v>
+      </x:c>
+      <x:c r="F7" s="155" t="str">
+        <x:v>Daily Production</x:v>
+      </x:c>
+      <x:c r="G7" s="155" t="str">
+        <x:v>certified</x:v>
+      </x:c>
+      <x:c r="H7" s="155" t="str">
+        <x:v>Is missing evidence distinct from zero?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="56" customHeight="1">
+      <x:c r="A8" s="155" t="str">
+        <x:v>TR-003</x:v>
+      </x:c>
+      <x:c r="B8" s="155" t="str">
+        <x:v>Machine event</x:v>
+      </x:c>
+      <x:c r="C8" s="155" t="str">
+        <x:v>18-minute downtime</x:v>
+      </x:c>
+      <x:c r="D8" s="155" t="str">
+        <x:v>Classify event + link machine</x:v>
+      </x:c>
+      <x:c r="E8" s="155" t="str">
+        <x:v>Downtime minutes</x:v>
+      </x:c>
+      <x:c r="F8" s="155" t="str">
+        <x:v>Weekly Downtime</x:v>
+      </x:c>
+      <x:c r="G8" s="155" t="str">
+        <x:v>read back</x:v>
+      </x:c>
+      <x:c r="H8" s="155" t="str">
+        <x:v>Does remote content match the candidate?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="56" customHeight="1">
+      <x:c r="A9" s="155" t="str">
+        <x:v>TR-004</x:v>
+      </x:c>
+      <x:c r="B9" s="155" t="str">
+        <x:v>Labor note</x:v>
+      </x:c>
+      <x:c r="C9" s="155" t="str">
+        <x:v>Shift context entered</x:v>
+      </x:c>
+      <x:c r="D9" s="155" t="str">
+        <x:v>Attach source lineage</x:v>
+      </x:c>
+      <x:c r="E9" s="155" t="str">
+        <x:v>Supervisor context</x:v>
+      </x:c>
+      <x:c r="F9" s="155" t="str">
+        <x:v>Shift Draft</x:v>
+      </x:c>
+      <x:c r="G9" s="155" t="str">
+        <x:v>human review</x:v>
+      </x:c>
+      <x:c r="H9" s="155" t="str">
+        <x:v>What operational context must be added?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="157" t="str">
+        <x:v>Inspection rule: an output may advance only when identity, source lineage, semantics, publication state, and readback evidence agree.</x:v>
+      </x:c>
+      <x:c r="B11" s="157"/>
+      <x:c r="C11" s="157"/>
+      <x:c r="D11" s="157"/>
+      <x:c r="E11" s="157"/>
+      <x:c r="F11" s="157"/>
+      <x:c r="G11" s="157"/>
+      <x:c r="H11" s="157"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A11:H11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="23" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Exception review - synthetic operator cases</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>Examples show what the system surfaces and what remains a human decision.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5" ht="38" customHeight="1">
+      <x:c r="A5" s="151" t="str">
+        <x:v>CASE</x:v>
+      </x:c>
+      <x:c r="B5" s="151" t="str">
+        <x:v>OBSERVED CONDITION</x:v>
+      </x:c>
+      <x:c r="C5" s="151" t="str">
+        <x:v>SYSTEM CLASSIFICATION</x:v>
+      </x:c>
+      <x:c r="D5" s="151" t="str">
+        <x:v>AUTOMATED BEHAVIOR</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="str">
+        <x:v>HUMAN REVIEW</x:v>
+      </x:c>
+      <x:c r="F5" s="151" t="str">
+        <x:v>WRITE AUTHORITY</x:v>
+      </x:c>
+      <x:c r="G5" s="151" t="str">
+        <x:v>SAFE OUTCOME</x:v>
+      </x:c>
+      <x:c r="H5" s="151" t="str">
+        <x:v>WHY IT MATTERS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="64" customHeight="1">
+      <x:c r="A6" s="155" t="str">
+        <x:v>EX-01</x:v>
+      </x:c>
+      <x:c r="B6" s="155" t="str">
+        <x:v>Required source absent</x:v>
+      </x:c>
+      <x:c r="C6" s="155" t="str">
+        <x:v>pending_source</x:v>
+      </x:c>
+      <x:c r="D6" s="155" t="str">
+        <x:v>Retain expected output; do not publish</x:v>
+      </x:c>
+      <x:c r="E6" s="155" t="str">
+        <x:v>Confirm source arrival or operational exception</x:v>
+      </x:c>
+      <x:c r="F6" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G6" s="155" t="str">
+        <x:v>Missing remains missing</x:v>
+      </x:c>
+      <x:c r="H6" s="155" t="str">
+        <x:v>Prevents invented zeros</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="64" customHeight="1">
+      <x:c r="A7" s="155" t="str">
+        <x:v>EX-02</x:v>
+      </x:c>
+      <x:c r="B7" s="155" t="str">
+        <x:v>Equivalent replay</x:v>
+      </x:c>
+      <x:c r="C7" s="155" t="str">
+        <x:v>exact_no_op</x:v>
+      </x:c>
+      <x:c r="D7" s="155" t="str">
+        <x:v>Compare governed material identity</x:v>
+      </x:c>
+      <x:c r="E7" s="155" t="str">
+        <x:v>No action unless context changed</x:v>
+      </x:c>
+      <x:c r="F7" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G7" s="155" t="str">
+        <x:v>Zero second write</x:v>
+      </x:c>
+      <x:c r="H7" s="155" t="str">
+        <x:v>Avoids duplicate versions</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="64" customHeight="1">
+      <x:c r="A8" s="155" t="str">
+        <x:v>EX-03</x:v>
+      </x:c>
+      <x:c r="B8" s="155" t="str">
+        <x:v>Write accepted; response lost</x:v>
+      </x:c>
+      <x:c r="C8" s="155" t="str">
+        <x:v>readback_pending</x:v>
+      </x:c>
+      <x:c r="D8" s="155" t="str">
+        <x:v>GET exact item; never repeat PUT</x:v>
+      </x:c>
+      <x:c r="E8" s="155" t="str">
+        <x:v>Review only if readback disagrees</x:v>
+      </x:c>
+      <x:c r="F8" s="155" t="str">
+        <x:v>GET only</x:v>
+      </x:c>
+      <x:c r="G8" s="155" t="str">
+        <x:v>Settle or fail closed</x:v>
+      </x:c>
+      <x:c r="H8" s="155" t="str">
+        <x:v>Bounds ambiguity</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="64" customHeight="1">
+      <x:c r="A9" s="155" t="str">
+        <x:v>EX-04</x:v>
+      </x:c>
+      <x:c r="B9" s="155" t="str">
+        <x:v>Contract or lineage drift</x:v>
+      </x:c>
+      <x:c r="C9" s="155" t="str">
+        <x:v>contract_refusal</x:v>
+      </x:c>
+      <x:c r="D9" s="155" t="str">
+        <x:v>Stop interpretation/publication</x:v>
+      </x:c>
+      <x:c r="E9" s="155" t="str">
+        <x:v>Investigate configuration or source change</x:v>
+      </x:c>
+      <x:c r="F9" s="155" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="G9" s="155" t="str">
+        <x:v>Explicit refusal</x:v>
+      </x:c>
+      <x:c r="H9" s="155" t="str">
+        <x:v>Prevents silent semantic drift</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="38" customHeight="1">
+      <x:c r="A11" s="159" t="str">
+        <x:v>Decision boundary: the platform prepares, classifies, and refuses. Supervisors and managers interpret context and choose operational action.</x:v>
+      </x:c>
+      <x:c r="B11" s="159"/>
+      <x:c r="C11" s="159"/>
+      <x:c r="D11" s="159"/>
+      <x:c r="E11" s="159"/>
+      <x:c r="F11" s="159"/>
+      <x:c r="G11" s="159"/>
+      <x:c r="H11" s="159"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="A11:H11"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="146" t="str">
+        <x:v>Impact model - editable assumptions</x:v>
+      </x:c>
+      <x:c r="B1" s="146"/>
+      <x:c r="C1" s="146"/>
+      <x:c r="D1" s="146"/>
+      <x:c r="E1" s="146"/>
+      <x:c r="F1" s="146"/>
+      <x:c r="G1" s="146"/>
+      <x:c r="H1" s="146"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="146"/>
+      <x:c r="B2" s="146"/>
+      <x:c r="C2" s="146"/>
+      <x:c r="D2" s="146"/>
+      <x:c r="E2" s="146"/>
+      <x:c r="F2" s="146"/>
+      <x:c r="G2" s="146"/>
+      <x:c r="H2" s="146"/>
+    </x:row>
+    <x:row r="3" ht="26" customHeight="1">
+      <x:c r="A3" s="148" t="str">
+        <x:v>Planning scenarios only. Inputs are editable; outputs are formulas, not booked results.</x:v>
+      </x:c>
+      <x:c r="B3" s="148"/>
+      <x:c r="C3" s="148"/>
+      <x:c r="D3" s="148"/>
+      <x:c r="E3" s="148"/>
+      <x:c r="F3" s="148"/>
+      <x:c r="G3" s="148"/>
+      <x:c r="H3" s="148"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="150" t="str">
+        <x:v>MODEL</x:v>
+      </x:c>
+      <x:c r="B5" s="150" t="str">
+        <x:v>INPUT</x:v>
+      </x:c>
+      <x:c r="C5" s="150" t="str">
+        <x:v>VALUE</x:v>
+      </x:c>
+      <x:c r="D5" s="150" t="str">
+        <x:v>UNIT</x:v>
+      </x:c>
+      <x:c r="F5" s="156" t="str">
+        <x:v>OUTPUT</x:v>
+      </x:c>
+      <x:c r="G5" s="156" t="str">
+        <x:v>FORMULA</x:v>
+      </x:c>
+      <x:c r="H5" s="156" t="str">
+        <x:v>RESULT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" customHeight="1">
+      <x:c r="A6" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B6" s="160" t="str">
+        <x:v>Supervisor hours/week</x:v>
+      </x:c>
+      <x:c r="C6" s="161" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D6" s="160" t="str">
+        <x:v>hours</x:v>
+      </x:c>
+      <x:c r="F6" s="163" t="str">
+        <x:v>Labor hours/year</x:v>
+      </x:c>
+      <x:c r="G6" s="169" t="str">
+        <x:v>(20 + 10) hours × 52 weeks</x:v>
+      </x:c>
+      <x:c r="H6" s="164" t="n">
+        <x:f>(C6+C7)*C8</x:f>
+        <x:v>1560</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" customHeight="1">
+      <x:c r="A7" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B7" s="160" t="str">
+        <x:v>Manager hours/week</x:v>
+      </x:c>
+      <x:c r="C7" s="161" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="D7" s="160" t="str">
+        <x:v>hours</x:v>
+      </x:c>
+      <x:c r="F7" s="163" t="str">
+        <x:v>Modeled labor value</x:v>
+      </x:c>
+      <x:c r="G7" s="169" t="str">
+        <x:v>Labor hours × $33.33/hour</x:v>
+      </x:c>
+      <x:c r="H7" s="165" t="n">
+        <x:f>H6*C9</x:f>
+        <x:v>51994.799999999996</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" customHeight="1">
+      <x:c r="A8" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B8" s="160" t="str">
+        <x:v>Weeks/year</x:v>
+      </x:c>
+      <x:c r="C8" s="161" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D8" s="160" t="str">
+        <x:v>weeks</x:v>
+      </x:c>
+      <x:c r="F8" s="163" t="str">
+        <x:v>Estimated retrieval reduction</x:v>
+      </x:c>
+      <x:c r="G8" s="169" t="str">
+        <x:v>(25 minutes - 2 minutes) ÷ 25 minutes</x:v>
+      </x:c>
+      <x:c r="H8" s="166" t="n">
+        <x:f>(C10-C11)/C10</x:f>
+        <x:v>0.92</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="160" t="str">
+        <x:v>Labor</x:v>
+      </x:c>
+      <x:c r="B9" s="160" t="str">
+        <x:v>Blended hourly value</x:v>
+      </x:c>
+      <x:c r="C9" s="161" t="n">
+        <x:v>33.33</x:v>
+      </x:c>
+      <x:c r="D9" s="160" t="str">
+        <x:v>$/hour</x:v>
+      </x:c>
+      <x:c r="F9" s="163" t="str">
+        <x:v>Production-unit opportunity</x:v>
+      </x:c>
+      <x:c r="G9" s="169" t="str">
+        <x:v>5 minutes ÷ 60 × 1,000 production units × 52.5 × 52</x:v>
+      </x:c>
+      <x:c r="H9" s="164" t="n">
+        <x:f>C12/60*C13*C14*C15</x:f>
+        <x:v>227500</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="160" t="str">
+        <x:v>Retrieval</x:v>
+      </x:c>
+      <x:c r="B10" s="160" t="str">
+        <x:v>Baseline search</x:v>
+      </x:c>
+      <x:c r="C10" s="161" t="n">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="D10" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="G10" s="170"/>
+    </x:row>
+    <x:row r="11" ht="36" customHeight="1">
+      <x:c r="A11" s="160" t="str">
+        <x:v>Retrieval</x:v>
+      </x:c>
+      <x:c r="B11" s="160" t="str">
+        <x:v>Bounded retrieval</x:v>
+      </x:c>
+      <x:c r="C11" s="161" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="D11" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+      <x:c r="F11" s="157" t="str">
+        <x:v>Contribution-margin opportunity</x:v>
+      </x:c>
+      <x:c r="G11" s="99" t="str">
+        <x:v>Production-unit opportunity × $0.90/unit</x:v>
+      </x:c>
+      <x:c r="H11" s="167" t="n">
+        <x:f>H9*C16</x:f>
+        <x:v>204750</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B12" s="160" t="str">
+        <x:v>Response improvement</x:v>
+      </x:c>
+      <x:c r="C12" s="161" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D12" s="160" t="str">
+        <x:v>minutes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="30" customHeight="1">
+      <x:c r="A13" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B13" s="160" t="str">
+        <x:v>Throughput</x:v>
+      </x:c>
+      <x:c r="C13" s="161" t="n">
+        <x:v>1000</x:v>
+      </x:c>
+      <x:c r="D13" s="160" t="str">
+        <x:v>production units/hour/machine</x:v>
+      </x:c>
+      <x:c r="F13" s="168" t="str">
+        <x:v>Limitations: representative time study, role-rate assumptions, event frequency, throughput, response improvement, and margin are scenario inputs. Outputs are not realized savings, guaranteed production, or autonomous outcomes.</x:v>
+      </x:c>
+      <x:c r="G13" s="168"/>
+      <x:c r="H13" s="168"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B14" s="160" t="str">
+        <x:v>Events/week</x:v>
+      </x:c>
+      <x:c r="C14" s="161" t="n">
+        <x:v>52.5</x:v>
+      </x:c>
+      <x:c r="D14" s="160" t="str">
+        <x:v>events</x:v>
+      </x:c>
+      <x:c r="F14" s="168"/>
+      <x:c r="G14" s="168"/>
+      <x:c r="H14" s="168"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B15" s="160" t="str">
+        <x:v>Weeks/year</x:v>
+      </x:c>
+      <x:c r="C15" s="161" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="D15" s="160" t="str">
+        <x:v>weeks</x:v>
+      </x:c>
+      <x:c r="F15" s="168"/>
+      <x:c r="G15" s="168"/>
+      <x:c r="H15" s="168"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="160" t="str">
+        <x:v>Downtime</x:v>
+      </x:c>
+      <x:c r="B16" s="160" t="str">
+        <x:v>Contribution margin</x:v>
+      </x:c>
+      <x:c r="C16" s="161" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="D16" s="160" t="str">
+        <x:v>$/unit</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="173" t="str">
+        <x:v>REVIEWED PRODUCTION-COUNT CONFORMANCE</x:v>
+      </x:c>
+      <x:c r="B18" s="173"/>
+      <x:c r="C18" s="173"/>
+      <x:c r="D18" s="173"/>
+      <x:c r="E18" s="173"/>
+      <x:c r="F18" s="173"/>
+      <x:c r="G18" s="173"/>
+      <x:c r="H18" s="173"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="177" t="str">
+        <x:v>EVIDENCE</x:v>
+      </x:c>
+      <x:c r="B19" s="177" t="str">
+        <x:v>CLASS</x:v>
+      </x:c>
+      <x:c r="C19" s="177" t="str">
+        <x:v>LEGACY BASELINE</x:v>
+      </x:c>
+      <x:c r="D19" s="177" t="str">
+        <x:v>SYSTEM RESULT</x:v>
+      </x:c>
+      <x:c r="E19" s="177" t="str">
+        <x:v>CHANGE</x:v>
+      </x:c>
+      <x:c r="F19" s="177" t="str">
+        <x:v>SCOPE</x:v>
+      </x:c>
+      <x:c r="G19" s="177" t="str">
+        <x:v>INTERPRETATION</x:v>
+      </x:c>
+      <x:c r="H19" s="177" t="str">
+        <x:v>LIMIT</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="62" customHeight="1">
+      <x:c r="A20" s="182" t="str">
+        <x:v>Required production-count schema</x:v>
+      </x:c>
+      <x:c r="B20" s="182" t="str">
+        <x:v>Reviewed observation</x:v>
+      </x:c>
+      <x:c r="C20" s="183" t="n">
+        <x:v>0.75</x:v>
+      </x:c>
+      <x:c r="D20" s="183" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="183" t="n">
+        <x:v>0.25</x:v>
+      </x:c>
+      <x:c r="F20" s="182" t="str">
+        <x:v>Approximately six months</x:v>
+      </x:c>
+      <x:c r="G20" s="182" t="str">
+        <x:v>About one in four legacy reports did not conform; every reviewed system output did</x:v>
+      </x:c>
+      <x:c r="H20" s="182" t="str">
+        <x:v>Sample-bound; exact N/date range retained privately</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H2"/>
+    <x:mergeCell ref="A3:H3"/>
+    <x:mergeCell ref="F13:H15"/>
+    <x:mergeCell ref="A18:H18"/>
+  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Align public case study and delivered assistant status
</commit_message>
<xml_diff>
--- a/public/synthetic-reliability-report.xlsx
+++ b/public/synthetic-reliability-report.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R1758a175ab2e41aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="Rbbea1f3cce644b42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="R14e0e7c24f8540be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant Evidence" sheetId="4" r:id="R120125a1c8dc4dde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R7d5b502e136348fd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R7b615ea87e7742b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R9ef09e9c48944bc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" r:id="R09eb9cc9cfc94f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recovery Trace" sheetId="2" r:id="R48b29b4980e5441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operational Use" sheetId="3" r:id="Rd9d5021ae4db4233"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reporting Assistant" sheetId="4" r:id="R07bf7b1e0f5443a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Lineage" sheetId="5" r:id="R64c3a1efa1df4566"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exception Review" sheetId="6" r:id="R3f30f29e7c654881"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Impact Model" sheetId="7" r:id="R2771b231b9574791"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,14 +19,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="5">
+  <x:numFmts count="6">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
     <x:numFmt numFmtId="203" formatCode="$#,##0"/>
     <x:numFmt numFmtId="204" formatCode="0%"/>
+    <x:numFmt numFmtId="205" formatCode="&quot;$&quot;#,##0"/>
   </x:numFmts>
-  <x:fonts count="27">
+  <x:fonts count="28">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -178,8 +179,13 @@
       <x:color rgb="FF171717"/>
       <x:name val="Aptos"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF333333"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="30">
+  <x:fills count="39">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -326,8 +332,53 @@
         <x:fgColor rgb="FFF4F4F2"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F1F1F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F1F1F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F1F1F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD52B1E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFBE8E6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="9">
+  <x:borders count="17">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -393,11 +444,87 @@
         <x:color rgb="FFD0D0CD"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFD0D0CD"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="184">
+  <x:cellXfs count="275">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -803,6 +930,189 @@
     </x:xf>
     <x:xf numFmtId="204" fontId="26" fillId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="32" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="32" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="32" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="27" fillId="32" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="35" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="35" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="35" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="27" fillId="35" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="38" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="27" fillId="38" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="38" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="205" fontId="27" fillId="38" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="27" fillId="38" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="18" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1783,7 +2093,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="127" t="str">
-        <x:v>Reporting Assistant — internal evidence and boundaries</x:v>
+        <x:v>Functional Reporting Assistant - evidence and boundaries</x:v>
       </x:c>
       <x:c r="B1" s="127"/>
       <x:c r="C1" s="127"/>
@@ -1803,51 +2113,51 @@
       <x:c r="G2" s="127"/>
       <x:c r="H2" s="127"/>
     </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="129" t="str">
-        <x:v>One public assistant; three controlled internal subsystems. Synthetic evidence only — no production connection or autonomous decisions.</x:v>
-      </x:c>
-      <x:c r="B3" s="129"/>
-      <x:c r="C3" s="129"/>
-      <x:c r="D3" s="129"/>
-      <x:c r="E3" s="129"/>
-      <x:c r="F3" s="129"/>
-      <x:c r="G3" s="129"/>
-      <x:c r="H3" s="129"/>
+    <x:row r="3" ht="38" customHeight="1">
+      <x:c r="A3" s="274" t="str">
+        <x:v>Delivered read-only extension: answers bounded, source-grounded queries with structured responses, validated citations, diagnostics, evidence validation, and deterministic refusal. Broader model-backed and advisory capabilities remain future work.</x:v>
+      </x:c>
+      <x:c r="B3" s="274"/>
+      <x:c r="C3" s="274"/>
+      <x:c r="D3" s="274"/>
+      <x:c r="E3" s="274"/>
+      <x:c r="F3" s="274"/>
+      <x:c r="G3" s="274"/>
+      <x:c r="H3" s="274"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="131" t="str">
         <x:v>SUBSYSTEM</x:v>
       </x:c>
-      <x:c r="B5" s="131" t="str"/>
+      <x:c r="B5" s="131"/>
       <x:c r="C5" s="131" t="str">
-        <x:v>CURRENT PURPOSE</x:v>
-      </x:c>
-      <x:c r="D5" s="131" t="str"/>
+        <x:v>FUNCTIONAL PURPOSE</x:v>
+      </x:c>
+      <x:c r="D5" s="131"/>
       <x:c r="E5" s="131" t="str">
         <x:v>VALIDATED BOUNDARY</x:v>
       </x:c>
-      <x:c r="F5" s="131" t="str"/>
+      <x:c r="F5" s="131"/>
       <x:c r="G5" s="131" t="str">
-        <x:v>VALUE SIGNAL</x:v>
+        <x:v>VALUE / FUTURE SIGNAL</x:v>
       </x:c>
       <x:c r="H5" s="131" t="str"/>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="135" t="str">
-        <x:v>Chatbot</x:v>
-      </x:c>
-      <x:c r="B6" s="135" t="str"/>
+        <x:v>Chatbot retrieval</x:v>
+      </x:c>
+      <x:c r="B6" s="135"/>
       <x:c r="C6" s="135" t="str">
-        <x:v>Source-grounded report retrieval</x:v>
-      </x:c>
-      <x:c r="D6" s="135" t="str"/>
+        <x:v>Answer bounded source-grounded queries</x:v>
+      </x:c>
+      <x:c r="D6" s="135"/>
       <x:c r="E6" s="135" t="str">
-        <x:v>Citations + deterministic fallback</x:v>
-      </x:c>
-      <x:c r="F6" s="135" t="str"/>
+        <x:v>Validated citations and deterministic fallback</x:v>
+      </x:c>
+      <x:c r="F6" s="135"/>
       <x:c r="G6" s="135" t="str">
-        <x:v>Estimated ~90% faster retrieval</x:v>
+        <x:v>Estimated ~90% retrieval scenario</x:v>
       </x:c>
       <x:c r="H6" s="135" t="str"/>
     </x:row>
@@ -1855,15 +2165,15 @@
       <x:c r="A7" s="135" t="str">
         <x:v>Report doctor</x:v>
       </x:c>
-      <x:c r="B7" s="135" t="str"/>
+      <x:c r="B7" s="135"/>
       <x:c r="C7" s="135" t="str">
         <x:v>Expected-output and exception diagnostics</x:v>
       </x:c>
-      <x:c r="D7" s="135" t="str"/>
+      <x:c r="D7" s="135"/>
       <x:c r="E7" s="135" t="str">
         <x:v>Read-only; no repair or publication</x:v>
       </x:c>
-      <x:c r="F7" s="135" t="str"/>
+      <x:c r="F7" s="135"/>
       <x:c r="G7" s="135" t="str">
         <x:v>Faster investigation</x:v>
       </x:c>
@@ -1873,23 +2183,23 @@
       <x:c r="A8" s="135" t="str">
         <x:v>Governed oracle</x:v>
       </x:c>
-      <x:c r="B8" s="135" t="str"/>
+      <x:c r="B8" s="135"/>
       <x:c r="C8" s="135" t="str">
-        <x:v>Contract-bound interpretation and validation</x:v>
-      </x:c>
-      <x:c r="D8" s="135" t="str"/>
+        <x:v>Contract-bound evidence validation</x:v>
+      </x:c>
+      <x:c r="D8" s="135"/>
       <x:c r="E8" s="135" t="str">
-        <x:v>Missing/ambiguous evidence fails closed</x:v>
-      </x:c>
-      <x:c r="F8" s="135" t="str"/>
+        <x:v>Missing or ambiguous evidence fails closed</x:v>
+      </x:c>
+      <x:c r="F8" s="135"/>
       <x:c r="G8" s="135" t="str">
         <x:v>Consistent evidence checks</x:v>
       </x:c>
       <x:c r="H8" s="135" t="str"/>
     </x:row>
-    <x:row r="10" ht="32" customHeight="1">
+    <x:row r="10" ht="42" customHeight="1">
       <x:c r="A10" s="143" t="str">
-        <x:v>Public materials present one Reporting Assistant; this technical sheet preserves internal subsystem names and boundaries.</x:v>
+        <x:v>Status boundary: the read-only assistant is functional and answers queries. It cannot write or publish reports or make operational decisions; broader model-backed reasoning, document knowledge, recurring artifacts, and advisory capabilities remain future work.</x:v>
       </x:c>
       <x:c r="B10" s="143"/>
       <x:c r="C10" s="143"/>
@@ -2377,14 +2687,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="22" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="15" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="40" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -2506,7 +2816,7 @@
         <x:v>weeks</x:v>
       </x:c>
       <x:c r="F8" s="163" t="str">
-        <x:v>Estimated retrieval reduction</x:v>
+        <x:v>Estimated assistant retrieval reduction</x:v>
       </x:c>
       <x:c r="G8" s="169" t="str">
         <x:v>(25 minutes - 2 minutes) ÷ 25 minutes</x:v>
@@ -2530,7 +2840,7 @@
         <x:v>$/hour</x:v>
       </x:c>
       <x:c r="F9" s="163" t="str">
-        <x:v>Production-unit opportunity</x:v>
+        <x:v>Machine-visibility production-unit opportunity</x:v>
       </x:c>
       <x:c r="G9" s="169" t="str">
         <x:v>5 minutes ÷ 60 × 1,000 production units × 52.5 × 52</x:v>
@@ -2542,7 +2852,7 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="160" t="str">
-        <x:v>Retrieval</x:v>
+        <x:v>Reporting Assistant</x:v>
       </x:c>
       <x:c r="B10" s="160" t="str">
         <x:v>Baseline search</x:v>
@@ -2553,11 +2863,12 @@
       <x:c r="D10" s="160" t="str">
         <x:v>minutes</x:v>
       </x:c>
+      <x:c r="F10"/>
       <x:c r="G10" s="170"/>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
       <x:c r="A11" s="160" t="str">
-        <x:v>Retrieval</x:v>
+        <x:v>Reporting Assistant</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
         <x:v>Bounded retrieval</x:v>
@@ -2569,7 +2880,7 @@
         <x:v>minutes</x:v>
       </x:c>
       <x:c r="F11" s="157" t="str">
-        <x:v>Contribution-margin opportunity</x:v>
+        <x:v>Machine-visibility contribution-margin opportunity</x:v>
       </x:c>
       <x:c r="G11" s="99" t="str">
         <x:v>Production-unit opportunity × $0.90/unit</x:v>
@@ -2581,7 +2892,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="160" t="str">
-        <x:v>Downtime</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B12" s="160" t="str">
         <x:v>Response improvement</x:v>
@@ -2595,7 +2906,7 @@
     </x:row>
     <x:row r="13" ht="30" customHeight="1">
       <x:c r="A13" s="160" t="str">
-        <x:v>Downtime</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B13" s="160" t="str">
         <x:v>Throughput</x:v>
@@ -2607,14 +2918,14 @@
         <x:v>production units/hour/machine</x:v>
       </x:c>
       <x:c r="F13" s="168" t="str">
-        <x:v>Limitations: representative time study, role-rate assumptions, event frequency, throughput, response improvement, and margin are scenario inputs. Outputs are not realized savings, guaranteed production, or autonomous outcomes.</x:v>
+        <x:v>Limitations: representative time study, role-rate assumptions, event frequency, throughput, response improvement, and margin are scenario inputs. The labor-capacity and machine-visibility value pools are separate and are not added together. Outputs are not realized savings, guaranteed production, or autonomous outcomes.</x:v>
       </x:c>
       <x:c r="G13" s="168"/>
       <x:c r="H13" s="168"/>
     </x:row>
     <x:row r="14" ht="30" customHeight="1">
       <x:c r="A14" s="160" t="str">
-        <x:v>Downtime</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B14" s="160" t="str">
         <x:v>Events/week</x:v>
@@ -2631,7 +2942,7 @@
     </x:row>
     <x:row r="15" ht="30" customHeight="1">
       <x:c r="A15" s="160" t="str">
-        <x:v>Downtime</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B15" s="160" t="str">
         <x:v>Weeks/year</x:v>
@@ -2648,7 +2959,7 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="160" t="str">
-        <x:v>Downtime</x:v>
+        <x:v>Machine visibility</x:v>
       </x:c>
       <x:c r="B16" s="160" t="str">
         <x:v>Contribution margin</x:v>
@@ -2660,75 +2971,130 @@
         <x:v>$/unit</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="30" customHeight="1">
-      <x:c r="A18" s="173" t="str">
-        <x:v>REVIEWED PRODUCTION-COUNT CONFORMANCE</x:v>
-      </x:c>
-      <x:c r="B18" s="173"/>
-      <x:c r="C18" s="173"/>
-      <x:c r="D18" s="173"/>
-      <x:c r="E18" s="173"/>
-      <x:c r="F18" s="173"/>
-      <x:c r="G18" s="173"/>
-      <x:c r="H18" s="173"/>
+    <x:row r="18" ht="24" customHeight="1">
+      <x:c r="A18" s="245" t="str">
+        <x:v>STATUS AND CLAIM BOUNDARIES</x:v>
+      </x:c>
+      <x:c r="B18" s="245"/>
+      <x:c r="C18" s="245"/>
+      <x:c r="D18" s="245"/>
+      <x:c r="E18" s="245"/>
+      <x:c r="F18" s="245"/>
+      <x:c r="G18" s="245"/>
+      <x:c r="H18" s="245"/>
     </x:row>
     <x:row r="19" ht="30" customHeight="1">
-      <x:c r="A19" s="177" t="str">
-        <x:v>EVIDENCE</x:v>
-      </x:c>
-      <x:c r="B19" s="177" t="str">
+      <x:c r="A19" s="248" t="str">
+        <x:v>AREA</x:v>
+      </x:c>
+      <x:c r="B19" s="248" t="str">
+        <x:v>STATUS</x:v>
+      </x:c>
+      <x:c r="C19" s="248" t="str">
+        <x:v>PRIMARY RESULT</x:v>
+      </x:c>
+      <x:c r="D19" s="248" t="str">
+        <x:v>UNIT</x:v>
+      </x:c>
+      <x:c r="E19" s="248" t="str">
+        <x:v>RELATED VALUE</x:v>
+      </x:c>
+      <x:c r="F19" s="248" t="str">
         <x:v>CLASS</x:v>
       </x:c>
-      <x:c r="C19" s="177" t="str">
-        <x:v>LEGACY BASELINE</x:v>
-      </x:c>
-      <x:c r="D19" s="177" t="str">
-        <x:v>SYSTEM RESULT</x:v>
-      </x:c>
-      <x:c r="E19" s="177" t="str">
-        <x:v>CHANGE</x:v>
-      </x:c>
-      <x:c r="F19" s="177" t="str">
-        <x:v>SCOPE</x:v>
-      </x:c>
-      <x:c r="G19" s="177" t="str">
-        <x:v>INTERPRETATION</x:v>
-      </x:c>
-      <x:c r="H19" s="177" t="str">
+      <x:c r="G19" s="248" t="str">
+        <x:v>SEPARATION</x:v>
+      </x:c>
+      <x:c r="H19" s="248" t="str">
         <x:v>LIMIT</x:v>
       </x:c>
     </x:row>
-    <x:row r="20" ht="62" customHeight="1">
-      <x:c r="A20" s="182" t="str">
-        <x:v>Required production-count schema</x:v>
-      </x:c>
-      <x:c r="B20" s="182" t="str">
-        <x:v>Reviewed observation</x:v>
-      </x:c>
-      <x:c r="C20" s="183" t="n">
-        <x:v>0.75</x:v>
-      </x:c>
-      <x:c r="D20" s="183" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="E20" s="183" t="n">
-        <x:v>0.25</x:v>
-      </x:c>
-      <x:c r="F20" s="182" t="str">
-        <x:v>Approximately six months</x:v>
-      </x:c>
-      <x:c r="G20" s="182" t="str">
-        <x:v>About one in four legacy reports did not conform; every reviewed system output did</x:v>
-      </x:c>
-      <x:c r="H20" s="182" t="str">
-        <x:v>Sample-bound; exact N/date range retained privately</x:v>
+    <x:row r="20" ht="46" customHeight="1">
+      <x:c r="A20" s="260" t="str">
+        <x:v>Core reporting</x:v>
+      </x:c>
+      <x:c r="B20" s="261" t="str">
+        <x:v>Delivered</x:v>
+      </x:c>
+      <x:c r="C20" s="269" t="n">
+        <x:f>'Impact Model'!H6</x:f>
+        <x:v>1560</x:v>
+      </x:c>
+      <x:c r="D20" s="261" t="str">
+        <x:v>hours/year</x:v>
+      </x:c>
+      <x:c r="E20" s="271" t="n">
+        <x:f>'Impact Model'!H7</x:f>
+        <x:v>51994.799999999996</x:v>
+      </x:c>
+      <x:c r="F20" s="261" t="str">
+        <x:v>Modeled labor-capacity value</x:v>
+      </x:c>
+      <x:c r="G20" s="261" t="str">
+        <x:v>Separate value pool</x:v>
+      </x:c>
+      <x:c r="H20" s="262" t="str">
+        <x:v>Not booked savings</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="46" customHeight="1">
+      <x:c r="A21" s="263" t="str">
+        <x:v>Machine visibility</x:v>
+      </x:c>
+      <x:c r="B21" s="264" t="str">
+        <x:v>Delivered extension</x:v>
+      </x:c>
+      <x:c r="C21" s="270" t="n">
+        <x:f>'Impact Model'!H9</x:f>
+        <x:v>227500</x:v>
+      </x:c>
+      <x:c r="D21" s="264" t="str">
+        <x:v>production units/year</x:v>
+      </x:c>
+      <x:c r="E21" s="272" t="n">
+        <x:f>'Impact Model'!H11</x:f>
+        <x:v>204750</x:v>
+      </x:c>
+      <x:c r="F21" s="264" t="str">
+        <x:v>Modeled upper bound</x:v>
+      </x:c>
+      <x:c r="G21" s="264" t="str">
+        <x:v>Separate value pool</x:v>
+      </x:c>
+      <x:c r="H21" s="265" t="str">
+        <x:v>Not realized production or margin</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="46" customHeight="1">
+      <x:c r="A22" s="266" t="str">
+        <x:v>Reporting Assistant</x:v>
+      </x:c>
+      <x:c r="B22" s="267" t="str">
+        <x:v>Delivered read-only extension</x:v>
+      </x:c>
+      <x:c r="C22" s="273" t="n">
+        <x:f>'Impact Model'!H8</x:f>
+        <x:v>0.92</x:v>
+      </x:c>
+      <x:c r="D22" s="267" t="str">
+        <x:v>retrieval reduction</x:v>
+      </x:c>
+      <x:c r="E22" s="267"/>
+      <x:c r="F22" s="267" t="str">
+        <x:v>Estimated scenario</x:v>
+      </x:c>
+      <x:c r="G22" s="267" t="str">
+        <x:v>Separate; not controlled benchmark</x:v>
+      </x:c>
+      <x:c r="H22" s="268" t="str">
+        <x:v>No write/advisory authority</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:H2"/>
     <x:mergeCell ref="A3:H3"/>
-    <x:mergeCell ref="F13:H15"/>
+    <x:mergeCell ref="F13:H16"/>
     <x:mergeCell ref="A18:H18"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>